<commit_message>
Act 1 banter polish: bail->debt reframe, Ch.8 clarity, plainer words
- bail -> debt everywhere (US-specific + off-theme for a pre-crime world;
  now universal and tied to Timely Rain's ledger). Ch.2/8/18/39 narration,
  Ch.2/19 banter. Ch.2 retitled "Bail Money" -> "Debt Paid".
- Ch.8: self-contained opener ("my old bosses sent me to rob you"), terse
  Li Kui closer, kept the witty Song Jiang line.
- Ch.3 "awning" -> "umbrella"; Ch.1 dragon joke on the visible tattoo.
Re-wired, rebuilt translations, re-exported web build.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Outer_Heaven_Reskin.xlsx
+++ b/Outer_Heaven_Reskin.xlsx
@@ -879,7 +879,7 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Bail Money</t>
+          <t>Debt Paid</t>
         </is>
       </c>
     </row>
@@ -1536,13 +1536,13 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Every child in the city learns the same bedtime story: a hundred and eight stars fall from heaven, live as heroes, and are called home when they die. Nine Dragons never believed it.
+          <t>Every child in the city learns the same bedtime story: a hundred and eight stars fall from heaven, live as heroes, and are called home when they die. Shi Jin never believed it.
 He believed in his job, his ink, and his morning noodles, until the Commission revised his future between two bites. Now there is a removal squad on the stairs, a stranger with a crossbow on the roof, and no path at all.</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Every child in the city learns the same bedtime story: a hundred and eight stars fall from heaven, live as heroes, and are called home when they die. Nine Dragons never believed it. He believed in his job, his ink, and his morning noodles, until the Commission revised his future between two bites. Now there is a removal squad on the stairs, a stranger with a crossbow on the roof, and no path at all.</t>
+          <t>Every child in the city learns the same bedtime story: a hundred and eight stars fall from heaven, live as heroes, and are called home when they die. Shi Jin never believed it. He believed in his job, his ink, and his morning noodles, until the Commission revised his future between two bites. Now there is a removal squad on the stairs, a stranger with a crossbow on the roof, and no path at all.</t>
         </is>
       </c>
     </row>
@@ -1552,19 +1552,19 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Bail Money</t>
+          <t>Debt Paid</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
           <t>The trains only stop where the Commission says the city exists. Everywhere else, people like Liu Tang carry what the trains will not: medicine, letters, other people's chances.
 This morning the system flagged his cargo as contraband and his temper as a crime in progress. Half right, as usual.
-He is heading for the one man who posts bail for strangers, and the crew is headed the same way.</t>
+He is heading for the one man who pays off strangers' debts, and the crew is headed the same way.</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>The trains only stop where the Commission says the city exists. Everywhere else, people like Liu Tang carry what the trains will not: medicine, letters, other people's chances. This morning the system flagged his cargo as contraband and his temper as a crime in progress. Half right, as usual. He is heading for the one man who posts bail for strangers, and the crew is headed the same way.</t>
+          <t>The trains only stop where the Commission says the city exists. Everywhere else, people like Liu Tang carry what the trains will not: medicine, letters, other people's chances. This morning the system flagged his cargo as contraband and his temper as a crime in progress. Half right, as usual. He is heading for the one man who pays off strangers' debts, and the crew is headed the same way.</t>
         </is>
       </c>
     </row>
@@ -1668,12 +1668,12 @@
       <c r="C8" s="7" t="inlineStr">
         <is>
           <t>The story about Lu Zhishen is that he hit an extortionist three times and the man stopped being alive. The story is true.
-He borrowed a monastery's robes on the way out, and the robes fit, more or less, the way vows do. Tonight a prison transport carries his new friend's teacher through the furnace district, and the Monk is standing in the road, cracking his knuckles at the headlights.</t>
+He borrowed a monastery's robes on the way out, and the robes fit, more or less, the way vows do. Tonight a prison transport rolls through the furnace district, packed with people flagged for nothing, and the Monk is already standing in the road, cracking his knuckles at the headlights.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>The story about Lu Zhishen is that he hit an extortionist three times and the man stopped being alive. The story is true. He borrowed a monastery's robes on the way out, and the robes fit, more or less, the way vows do. Tonight a prison transport carries his new friend's teacher through the furnace district, and the Monk is standing in the road, cracking his knuckles at the headlights.</t>
+          <t>The story about Lu Zhishen is that he hit an extortionist three times and the man stopped being alive. The story is true. He borrowed a monastery's robes on the way out, and the robes fit, more or less, the way vows do. Tonight a prison transport rolls through the furnace district, packed with people flagged for nothing, and the Monk is already standing in the road, cracking his knuckles at the headlights.</t>
         </is>
       </c>
     </row>
@@ -1689,13 +1689,13 @@
       <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Li Kui repossesses things for a living: cars, machines, once an entire carousel. Strongest hands in the undercity, no record of ever using them on a person.
-Today's work order says: the bail office by the lake, everything inside, the ledger too. Li Kui reads slowly.
+Today's work order says: the office by the lake that clears debts, everything inside, the ledger too. Li Kui reads slowly.
 Then he reads who signed it. Then he brings the work order back to the depot, in pieces, for filing.</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Li Kui repossesses things for a living: cars, machines, once an entire carousel. Strongest hands in the undercity, no record of ever using them on a person. Today's work order says: the bail office by the lake, everything inside, the ledger too. Li Kui reads slowly. Then he reads who signed it. Then he brings the work order back to the depot, in pieces, for filing.</t>
+          <t>Li Kui repossesses things for a living: cars, machines, once an entire carousel. Strongest hands in the undercity, no record of ever using them on a person. Today's work order says: the office by the lake that clears debts, everything inside, the ledger too. Li Kui reads slowly. Then he reads who signed it. Then he brings the work order back to the depot, in pieces, for filing.</t>
         </is>
       </c>
     </row>
@@ -1908,14 +1908,14 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>The order goes out to every range-master in the city: on sight, Timely Rain, lethal authorization. Hua Rong grew up on that man's bail money.
+          <t>The order goes out to every range-master in the city: on sight, Timely Rain, lethal authorization. Hua Rong grew up on debts that man quietly paid.
 He files his refusal the loud way, from four hundred meters, past three officers' hats and through the warrant sheet pinned to the wall. Nobody is hurt.
 Everybody is informed. The finest shot in the Commission's ranks would like Outer Heaven to know he is coming, and he brings his own bow.</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>The order goes out to every range-master in the city: on sight, Timely Rain, lethal authorization. Hua Rong grew up on that man's bail money. He files his refusal the loud way, from four hundred meters, past three officers' hats and through the warrant sheet pinned to the wall. Nobody is hurt. Everybody is informed. The finest shot in the Commission's ranks would like Outer Heaven to know he is coming, and he brings his own bow.</t>
+          <t>The order goes out to every range-master in the city: on sight, Timely Rain, lethal authorization. Hua Rong grew up on debts that man quietly paid. He files his refusal the loud way, from four hundred meters, past three officers' hats and through the warrant sheet pinned to the wall. Nobody is hurt. Everybody is informed. The finest shot in the Commission's ranks would like Outer Heaven to know he is coming, and he brings his own bow.</t>
         </is>
       </c>
     </row>
@@ -2169,12 +2169,12 @@
         <is>
           <t>The city starts talking back. Thank-you notes on the park fence, soup left at the gate, a mural of a tiger nobody will admit painting.
 And down from the hills comes a hunter with beast-sign maps a year deep: the monsters are not wandering, they are being herded, driven along survey lines toward wherever Deviants gather. Somebody is aiming the wilderness.
-Two-Headed Snake wants to know who, and his sister is already tracking.</t>
+Xie Zhen, the Two-Headed Snake, wants to know who, and his sister is already tracking.</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>The city starts talking back. Thank-you notes on the park fence, soup left at the gate, a mural of a tiger nobody will admit painting. And down from the hills comes a hunter with beast-sign maps a year deep: the monsters are not wandering, they are being herded, driven along survey lines toward wherever Deviants gather. Somebody is aiming the wilderness. Two-Headed Snake wants to know who, and his sister is already tracking.</t>
+          <t>The city starts talking back. Thank-you notes on the park fence, soup left at the gate, a mural of a tiger nobody will admit painting. And down from the hills comes a hunter with beast-sign maps a year deep: the monsters are not wandering, they are being herded, driven along survey lines toward wherever Deviants gather. Somebody is aiming the wilderness. Xie Zhen, the Two-Headed Snake, wants to know who, and his sister is already tracking.</t>
         </is>
       </c>
     </row>
@@ -2190,13 +2190,13 @@
       <c r="C32" s="7" t="inlineStr">
         <is>
           <t>The mountain has a king: an old horned beast that never once came below the tree line, until a Commission survey barge parked over its den and started pinging. Maddened, it comes down on the crew like weather.
-Twin-Tailed Scorpion drops out of a pine mid-sentence, finishing one her brother started a week ago, and between the two of them the hunt turns. The beast dies angry.
+Xie Bao, the Twin-Tailed Scorpion, drops out of a pine mid-sentence, finishing one her brother started a week ago, and between the two of them the hunt turns. The beast dies angry.
 The barge, they notice, was never armed. It was measuring.</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>The mountain has a king: an old horned beast that never once came below the tree line, until a Commission survey barge parked over its den and started pinging. Maddened, it comes down on the crew like weather. Twin-Tailed Scorpion drops out of a pine mid-sentence, finishing one her brother started a week ago, and between the two of them the hunt turns. The beast dies angry. The barge, they notice, was never armed. It was measuring.</t>
+          <t>The mountain has a king: an old horned beast that never once came below the tree line, until a Commission survey barge parked over its den and started pinging. Maddened, it comes down on the crew like weather. Xie Bao, the Twin-Tailed Scorpion, drops out of a pine mid-sentence, finishing one her brother started a week ago, and between the two of them the hunt turns. The beast dies angry. The barge, they notice, was never armed. It was measuring.</t>
         </is>
       </c>
     </row>
@@ -2302,13 +2302,12 @@
         <is>
           <t>The Southbank campaign opens exactly as briefed, which should be the first warning. Every bridge falls on schedule.
 Every ambush is pre-cleared. The crew wins and wins and feels like a hand inside a glove inside a fist.
-Today's orders: the third bridge. Hold it four minutes so the families can cross.
-Fiery Thunderbolt volunteers before anyone finishes reading. Bridges, he says, are honest work.</t>
+Then comes an order with a hero-sized hole in it: one span, held to the second, so two families can slip across. Fiery Thunderbolt volunteers before the briefing even ends.</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>The Southbank campaign opens exactly as briefed, which should be the first warning. Every bridge falls on schedule. Every ambush is pre-cleared. The crew wins and wins and feels like a hand inside a glove inside a fist. Today's orders: the third bridge. Hold it four minutes so the families can cross. Fiery Thunderbolt volunteers before anyone finishes reading. Bridges, he says, are honest work.</t>
+          <t>The Southbank campaign opens exactly as briefed, which should be the first warning. Every bridge falls on schedule. Every ambush is pre-cleared. The crew wins and wins and feels like a hand inside a glove inside a fist. Then comes an order with a hero-sized hole in it: one span, held to the second, so two families can slip across. Fiery Thunderbolt volunteers before the briefing even ends.</t>
         </is>
       </c>
     </row>
@@ -2370,12 +2369,12 @@
         <is>
           <t>Ascension Day. The tower opens like a church.
 Below the last floor there is no machine, no god, no code: jars. Rows of old minds in warm fluid, watching through the walls, and a recording in the founder's own voice, practicing the star legend until it sounded kind.
-On a screen a life plays back: a clerk who always had bail money, built kindness by kindness to gather the best. Timely Rain watches his whole self turn into handwriting.</t>
+On a screen a life plays back: a clerk who always had money for someone else's debt, built kindness by kindness to gather the best. Timely Rain watches his whole self turn into handwriting.</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Ascension Day. The tower opens like a church. Below the last floor there is no machine, no god, no code: jars. Rows of old minds in warm fluid, watching through the walls, and a recording in the founder's own voice, practicing the star legend until it sounded kind. On a screen a life plays back: a clerk who always had bail money, built kindness by kindness to gather the best. Timely Rain watches his whole self turn into handwriting.</t>
+          <t>Ascension Day. The tower opens like a church. Below the last floor there is no machine, no god, no code: jars. Rows of old minds in warm fluid, watching through the walls, and a recording in the founder's own voice, practicing the star legend until it sounded kind. On a screen a life plays back: a clerk who always had money for someone else's debt, built kindness by kindness to gather the best. Timely Rain watches his whole self turn into handwriting.</t>
         </is>
       </c>
     </row>
@@ -22123,7 +22122,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>You have nine, and they're all dragons. Move.</t>
+          <t>You've got nine dragons inked up your arms. That's name enough. Move.</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -22133,7 +22132,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>You have nine, and they're all dragons. Move.</t>
+          <t>You've got nine dragons inked up your arms. That's name enough. Move.</t>
         </is>
       </c>
     </row>
@@ -22147,7 +22146,7 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Pin it, break it, nobody bleed. I left my good thread at home.</t>
+          <t>I'm a doctor, not backup. If anyone bleeds today, it had better be the drone.</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -22157,7 +22156,7 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>Pin it, break it, nobody bleed. I left my good thread at home.</t>
+          <t>I'm a doctor, not backup. If anyone bleeds today, it had better be the drone.</t>
         </is>
       </c>
     </row>
@@ -22167,7 +22166,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Bail Money</t>
+          <t>Debt Paid</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -22177,7 +22176,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>You three following me? I bite, and I owe bail money.</t>
+          <t>Stop following me. I bite, and I'm already buried in debt.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -22187,7 +22186,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>You three following me? I bite, and I owe bail money.</t>
+          <t>Stop following me. I bite, and I'm already buried in debt.</t>
         </is>
       </c>
     </row>
@@ -22201,7 +22200,7 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Everyone we like owes bail money. Who's your bondsman?</t>
+          <t>Everyone we like is buried in debt. Who paid yours?</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -22211,7 +22210,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Everyone we like owes bail money. Who's your bondsman?</t>
+          <t>Everyone we like is buried in debt. Who paid yours?</t>
         </is>
       </c>
     </row>
@@ -22225,7 +22224,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Man called Timely Rain. Never met him. He paid anyway.</t>
+          <t>Man called Timely Rain. Never met him. He paid it off anyway.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -22235,7 +22234,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Man called Timely Rain. Never met him. He paid anyway.</t>
+          <t>Man called Timely Rain. Never met him. He paid it off anyway.</t>
         </is>
       </c>
     </row>
@@ -22249,7 +22248,7 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>A stranger who pays? Now I've heard folklore.</t>
+          <t>A stranger who clears your debt? Now I've heard folklore.</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -22259,7 +22258,7 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>A stranger who pays? Now I've heard folklore.</t>
+          <t>A stranger who clears your debt? Now I've heard folklore.</t>
         </is>
       </c>
     </row>
@@ -22279,7 +22278,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>You'll want the awning in forty seconds. Also, the big one flanks left.</t>
+          <t>You'll want an umbrella in forty seconds. Also, the big one flanks left.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -22289,7 +22288,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>You'll want the awning in forty seconds. Also, the big one flanks left.</t>
+          <t>You'll want an umbrella in forty seconds. Also, the big one flanks left.</t>
         </is>
       </c>
     </row>
@@ -22657,7 +22656,7 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Ninety-four percent. That's what they think of me.</t>
+          <t>They took the school. My rank. Her. I raised no hand. The file did it all.</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -22667,7 +22666,7 @@
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Ninety-four percent. That's what they think of me.</t>
+          <t>They took the school. My rank. Her. I raised no hand. The file did it all.</t>
         </is>
       </c>
     </row>
@@ -22681,7 +22680,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>I'm a twelve. Flight risk, not fight risk. We average out nicely.</t>
+          <t>A file did that in a day? Then the Commission's the disease. Not you.</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -22691,7 +22690,7 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>I'm a twelve. Flight risk, not fight risk. We average out nicely.</t>
+          <t>A file did that in a day? Then the Commission's the disease. Not you.</t>
         </is>
       </c>
     </row>
@@ -22783,7 +22782,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Twelve. And dropping, thanks to present company.</t>
+          <t>Twelve. Apparently I'm a flight risk, not a fight risk.</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
@@ -22793,7 +22792,7 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>Twelve. And dropping, thanks to present company.</t>
+          <t>Twelve. Apparently I'm a flight risk, not a fight risk.</t>
         </is>
       </c>
     </row>
@@ -22807,7 +22806,7 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>She's still in the city. And I'm here.</t>
+          <t>My wife is still in the city. I'm down here. That's the score.</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -22817,7 +22816,7 @@
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>She's still in the city. And I'm here.</t>
+          <t>My wife is still in the city. I'm down here. That's the score.</t>
         </is>
       </c>
     </row>
@@ -22861,7 +22860,7 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>New plan. We hit the depot until it apologizes.</t>
+          <t>My old bosses sent me to rob you. New plan: we go make them apologize. With hammers.</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -22871,7 +22870,7 @@
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>New plan. We hit the depot until it apologizes.</t>
+          <t>My old bosses sent me to rob you. New plan: we go make them apologize. With hammers.</t>
         </is>
       </c>
     </row>
@@ -22957,7 +22956,7 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>No promises. One promise. That one.</t>
+          <t>I'll try. For you. Nobody else.</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -22967,7 +22966,7 @@
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>No promises. One promise. That one.</t>
+          <t>I'll try. For you. Nobody else.</t>
         </is>
       </c>
     </row>
@@ -24127,7 +24126,7 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Then we drill today. Nobody dies rescuing the man who bailed us out. He'd hate the math.</t>
+          <t>Then we drill today. Nobody dies rescuing the man who cleared our debts. He'd hate the math.</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
@@ -24137,7 +24136,7 @@
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>Then we drill today. Nobody dies rescuing the man who bailed us out. He'd hate the math.</t>
+          <t>Then we drill today. Nobody dies rescuing the man who cleared our debts. He'd hate the math.</t>
         </is>
       </c>
     </row>
@@ -25021,7 +25020,7 @@
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>Don't. Whatever you're going to say, the tiger heard it first.</t>
+          <t>Don't say it. I know how this road ends. I walked it for my brother.</t>
         </is>
       </c>
       <c r="E118" s="6" t="inlineStr">
@@ -25031,7 +25030,7 @@
       </c>
       <c r="F118" s="7" t="inlineStr">
         <is>
-          <t>Don't. Whatever you're going to say, the tiger heard it first.</t>
+          <t>Don't say it. I know how this road ends. I walked it for my brother.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enemy naming overhaul + kill phantom-duel narration
- reskin_enemy(): 51 enemies that fell through to "Stray Beast" now get
  thematic names via keyword matching - rebels->Southbank, mechanical
  names->Enforcement/Arc/Works Machine, nega->the Hollow, plus Horned/
  Sky/Shell/Blade/Frost/Fen beast families. Fallback is "Undercity Beast".
  Signature bosses keep their BOSS-dict names where TB places them
  (Flawless One Ch34, Council Wardens, Xaepha, Defector Frame). 0 generics.
- reskin_appearance(): matching one-line looks for every new family.
- Ch.16/17 narration: reframed so you break his forces (sentinels/columns)
  instead of claiming a personal duel the battle doesn't stage.
Re-wired names+descriptions+narration, reimported, re-exported. Suite green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Outer_Heaven_Reskin.xlsx
+++ b/Outer_Heaven_Reskin.xlsx
@@ -1872,7 +1872,7 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>The Commission answers the heist with its favorite hammer: Qin Ming, garrison champion, a man whose temper arrives before his orders do. The Wisdom Star baits him into the flood channels, beats him fair, and sends him home embarrassed. He gets there in time to watch the Commission burn his garrison for the crime of losing. They wrote him off as a failure, so they billed him the fire. He walks back to Outer Heaven carrying the ashes and his mace.</t>
+          <t>The Commission answers the heist with its favorite hammer: Qin Ming, garrison champion, a man whose temper arrives before his orders do. The Wisdom Star baits his overcharged sentinels into the flood channels and shorts them out, one by one, until the champion is left commanding nothing but sparks. He gets home in time to watch the Commission burn that garrison for the crime of losing. They wrote him off as a failure, so they billed him the fire. He walks back to Outer Heaven carrying the ashes and his mace.</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Marshal Huyan Zhuo does not lose, and the Commission sends him to prove it. He comes down the lake road with armor columns and a career of medals, and Outer Heaven holds. Beaten fair, he asks for a rematch. Then, on his way out, he passes an enforcement squad burning a food line for the crime of feeding Deviants, and something in the marshal finishes changing sides before the rematch does.</t>
+          <t>Marshal Huyan Zhuo does not lose, and the Commission sends him to prove it. He comes down the lake road with armor columns and a career of medals, and the columns break against Outer Heaven's walls. Beaten for the first time in that career, he asks for a rematch. Then, on his way out, he passes an enforcement squad burning a food line for the crime of feeding Deviants, and something in the marshal finishes changing sides before the rematch does.</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Council Warden, Lesser</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A lesser tower guardian, unfinished but lethal, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Council Warden, Lesser</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A lesser tower guardian, unfinished but lethal, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Council Warden, Lesser</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A lesser tower guardian, unfinished but lethal, a long pike.</t>
         </is>
       </c>
     </row>
@@ -3795,7 +3795,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Council Warden, Lesser</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A lesser tower guardian, unfinished but lethal, a long pike.</t>
         </is>
       </c>
     </row>
@@ -3847,7 +3847,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Council Warden, Lesser</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A lesser tower guardian, unfinished but lethal, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Council Warden, Lesser</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="L7" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A lesser tower guardian, unfinished but lethal, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -3991,7 +3991,7 @@
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A beast of the undercity, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Iron Crawler</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -4043,7 +4043,7 @@
       </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A many-legged iron crawler that skitters along the walls, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4107,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Enforcement Machine</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a long pike.</t>
+          <t>A heavy Commission war-machine, servos hissing, frost-rimed a long pike.</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -4195,7 +4195,7 @@
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A beast of the undercity, bare claws.</t>
         </is>
       </c>
     </row>
@@ -4207,7 +4207,7 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A beast of the undercity, bare claws.</t>
         </is>
       </c>
     </row>
@@ -4307,7 +4307,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="L15" s="9" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a charged rod.</t>
+          <t>A frost-rimed beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Blade Beast</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A lean cutthroat shape all edges, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Blade Beast</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="L21" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A lean cutthroat shape all edges, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Horned Beast</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -4711,7 +4711,7 @@
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A heavy horned beast of the old wilds, a long pike.</t>
         </is>
       </c>
     </row>
@@ -4723,7 +4723,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A beast of the undercity, a long pike.</t>
         </is>
       </c>
     </row>
@@ -5087,7 +5087,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A beast of the undercity, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Arc Machine</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a charged rod.</t>
+          <t>A crackling Commission unit sheathed in live current, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -5279,7 +5279,7 @@
       </c>
       <c r="L33" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A beast of the undercity, bare claws.</t>
         </is>
       </c>
     </row>
@@ -5395,7 +5395,7 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A beast of the undercity, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -5447,7 +5447,7 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
@@ -5487,7 +5487,7 @@
       </c>
       <c r="L37" s="9" t="inlineStr">
         <is>
-          <t>A flame-scarred stray beast of the undercity, a charged rod.</t>
+          <t>A flame-scarred beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -5499,7 +5499,7 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -5539,7 +5539,7 @@
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A beast of the undercity, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="L39" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -5707,7 +5707,7 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>A night-black stray beast of the undercity, a charged rod.</t>
+          <t>A night-black beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -5759,7 +5759,7 @@
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Frost Beast</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="L43" s="9" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a heavy blade.</t>
+          <t>A hunched beast rimed in lake ice, breath like winter, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -5863,7 +5863,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Frost Beast</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="L45" s="9" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a charged rod.</t>
+          <t>A hunched beast rimed in lake ice, breath like winter, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -5915,7 +5915,7 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Frost Beast</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
@@ -5955,7 +5955,7 @@
       </c>
       <c r="L46" s="7" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a long pike.</t>
+          <t>A hunched beast rimed in lake ice, breath like winter, a long pike.</t>
         </is>
       </c>
     </row>
@@ -5967,7 +5967,7 @@
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Frost Beast</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="L47" s="9" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a charged rod.</t>
+          <t>A hunched beast rimed in lake ice, breath like winter, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -6019,7 +6019,7 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Blade Beast</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="L48" s="7" t="inlineStr">
         <is>
-          <t>A night-black stray beast of the undercity, a heavy blade.</t>
+          <t>A lean cutthroat shape all edges, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -6071,7 +6071,7 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Enforcement Machine</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="L49" s="9" t="inlineStr">
         <is>
-          <t>A flame-scarred stray beast of the undercity, a heavy blade.</t>
+          <t>A heavy Commission war-machine, servos hissing, flame-scarred a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Enforcement Machine</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
@@ -6215,7 +6215,7 @@
       </c>
       <c r="L51" s="9" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a long pike.</t>
+          <t>A heavy Commission war-machine, servos hissing, storm-lit a long pike.</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
@@ -6475,7 +6475,7 @@
       </c>
       <c r="L56" s="7" t="inlineStr">
         <is>
-          <t>A night-black stray beast of the undercity, a charged rod.</t>
+          <t>A night-black beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
@@ -6527,7 +6527,7 @@
       </c>
       <c r="L57" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A beast of the undercity, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -6539,7 +6539,7 @@
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Arc Machine</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
@@ -6579,7 +6579,7 @@
       </c>
       <c r="L58" s="7" t="inlineStr">
         <is>
-          <t>A night-black stray beast of the undercity, a long pike.</t>
+          <t>A crackling Commission unit sheathed in live current, a long pike.</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Shell Beast</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
@@ -6631,7 +6631,7 @@
       </c>
       <c r="L59" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A slab-shelled beast that shrugs off blows, a long pike.</t>
         </is>
       </c>
     </row>
@@ -6695,7 +6695,7 @@
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Force Node</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="L61" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A floating node that hardens everything around it; break it first.</t>
         </is>
       </c>
     </row>
@@ -6747,7 +6747,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Sky Beast</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
@@ -6787,7 +6787,7 @@
       </c>
       <c r="L62" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A winged thing out of the reactor haze, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -6799,7 +6799,7 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>the Hollow</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="L63" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A walking piece of absence, eating color and sound, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -6903,7 +6903,7 @@
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="L65" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A beast of the undercity, a long pike.</t>
         </is>
       </c>
     </row>
@@ -6955,7 +6955,7 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Arc Machine</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
@@ -6995,7 +6995,7 @@
       </c>
       <c r="L66" s="7" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a compound bow.</t>
+          <t>A crackling Commission unit sheathed in live current, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -7007,7 +7007,7 @@
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Arc Machine</t>
         </is>
       </c>
       <c r="C67" s="9" t="inlineStr">
@@ -7047,7 +7047,7 @@
       </c>
       <c r="L67" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A crackling Commission unit sheathed in live current, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -7059,7 +7059,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Arc Machine</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
@@ -7099,7 +7099,7 @@
       </c>
       <c r="L68" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A crackling Commission unit sheathed in live current, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -7111,7 +7111,7 @@
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Arc Machine</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
@@ -7151,7 +7151,7 @@
       </c>
       <c r="L69" s="9" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a heavy blade.</t>
+          <t>A crackling Commission unit sheathed in live current, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -7163,7 +7163,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Arc Machine</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
@@ -7203,7 +7203,7 @@
       </c>
       <c r="L70" s="7" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a long pike.</t>
+          <t>A crackling Commission unit sheathed in live current, a long pike.</t>
         </is>
       </c>
     </row>
@@ -7215,7 +7215,7 @@
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C71" s="9" t="inlineStr">
@@ -7255,7 +7255,7 @@
       </c>
       <c r="L71" s="9" t="inlineStr">
         <is>
-          <t>A flame-scarred stray beast of the undercity, a charged rod.</t>
+          <t>A flame-scarred beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -7267,7 +7267,7 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="L72" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -7319,7 +7319,7 @@
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Fen Spirit</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr">
@@ -7359,7 +7359,7 @@
       </c>
       <c r="L73" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A marsh-wisp of the drowned undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -7423,7 +7423,7 @@
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr">
@@ -7459,7 +7459,7 @@
       </c>
       <c r="L75" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A beast of the undercity, bare claws.</t>
         </is>
       </c>
     </row>
@@ -7627,7 +7627,7 @@
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Iron Crawler</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
@@ -7667,7 +7667,7 @@
       </c>
       <c r="L79" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A many-legged iron crawler that skitters along the walls, a long pike.</t>
         </is>
       </c>
     </row>
@@ -7679,7 +7679,7 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
@@ -7719,7 +7719,7 @@
       </c>
       <c r="L80" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -7731,7 +7731,7 @@
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Frost Beast</t>
         </is>
       </c>
       <c r="C81" s="9" t="inlineStr">
@@ -7771,7 +7771,7 @@
       </c>
       <c r="L81" s="9" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a long pike.</t>
+          <t>A hunched beast rimed in lake ice, breath like winter, a long pike.</t>
         </is>
       </c>
     </row>
@@ -7835,7 +7835,7 @@
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Sky Beast</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="L83" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A winged thing out of the reactor haze, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
@@ -7927,7 +7927,7 @@
       </c>
       <c r="L84" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A beast of the undercity, a long pike.</t>
         </is>
       </c>
     </row>
@@ -7939,7 +7939,7 @@
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C85" s="9" t="inlineStr">
@@ -7975,7 +7975,7 @@
       </c>
       <c r="L85" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A beast of the undercity, bare claws.</t>
         </is>
       </c>
     </row>
@@ -7987,7 +7987,7 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Horned Beast</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
@@ -8027,7 +8027,7 @@
       </c>
       <c r="L86" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A heavy horned beast of the old wilds, a long pike.</t>
         </is>
       </c>
     </row>
@@ -8039,7 +8039,7 @@
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C87" s="9" t="inlineStr">
@@ -8079,7 +8079,7 @@
       </c>
       <c r="L87" s="9" t="inlineStr">
         <is>
-          <t>A flame-scarred stray beast of the undercity, a charged rod.</t>
+          <t>A flame-scarred beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -8091,7 +8091,7 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Enforcement Machine</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="L88" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A heavy Commission war-machine, servos hissing, bare claws.</t>
         </is>
       </c>
     </row>
@@ -8175,7 +8175,7 @@
       </c>
       <c r="L89" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A beast of the undercity, bare claws.</t>
         </is>
       </c>
     </row>
@@ -8239,7 +8239,7 @@
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C91" s="9" t="inlineStr">
@@ -8279,7 +8279,7 @@
       </c>
       <c r="L91" s="9" t="inlineStr">
         <is>
-          <t>A night-black stray beast of the undercity, a charged rod.</t>
+          <t>A night-black beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -8291,7 +8291,7 @@
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Sky Beast</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
@@ -8331,7 +8331,7 @@
       </c>
       <c r="L92" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A winged thing out of the reactor haze, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -8395,7 +8395,7 @@
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Sky Beast</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
@@ -8435,7 +8435,7 @@
       </c>
       <c r="L94" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A winged thing out of the reactor haze, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -8499,7 +8499,7 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
@@ -8539,7 +8539,7 @@
       </c>
       <c r="L96" s="7" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a charged rod.</t>
+          <t>A storm-lit beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -8863,7 +8863,7 @@
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C103" s="9" t="inlineStr">
@@ -8903,7 +8903,7 @@
       </c>
       <c r="L103" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A beast of the undercity, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -8915,7 +8915,7 @@
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Enforcement Machine</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="L104" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A heavy Commission war-machine, servos hissing, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -8967,7 +8967,7 @@
       </c>
       <c r="B105" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Horned Beast</t>
         </is>
       </c>
       <c r="C105" s="9" t="inlineStr">
@@ -9007,7 +9007,7 @@
       </c>
       <c r="L105" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A heavy horned beast of the old wilds, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -9019,7 +9019,7 @@
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
@@ -9059,7 +9059,7 @@
       </c>
       <c r="L106" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A beast of the undercity, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -9071,7 +9071,7 @@
       </c>
       <c r="B107" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Enforcement Machine</t>
         </is>
       </c>
       <c r="C107" s="9" t="inlineStr">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="L107" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A heavy Commission war-machine, servos hissing, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -9123,7 +9123,7 @@
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Enforcement Machine</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
@@ -9163,7 +9163,7 @@
       </c>
       <c r="L108" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A heavy Commission war-machine, servos hissing, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -9175,7 +9175,7 @@
       </c>
       <c r="B109" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C109" s="9" t="inlineStr">
@@ -9215,7 +9215,7 @@
       </c>
       <c r="L109" s="9" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a charged rod.</t>
+          <t>A frost-rimed beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -9227,7 +9227,7 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Fen Spirit</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
@@ -9267,7 +9267,7 @@
       </c>
       <c r="L110" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A marsh-wisp of the drowned undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -9279,7 +9279,7 @@
       </c>
       <c r="B111" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Creeper</t>
         </is>
       </c>
       <c r="C111" s="9" t="inlineStr">
@@ -9319,7 +9319,7 @@
       </c>
       <c r="L111" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A low creeping horror that hugs the ground, a long pike.</t>
         </is>
       </c>
     </row>
@@ -9695,7 +9695,7 @@
       </c>
       <c r="B119" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C119" s="9" t="inlineStr">
@@ -9735,7 +9735,7 @@
       </c>
       <c r="L119" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -9951,7 +9951,7 @@
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Sludge Beast</t>
         </is>
       </c>
       <c r="C124" s="7" t="inlineStr">
@@ -9991,7 +9991,7 @@
       </c>
       <c r="L124" s="7" t="inlineStr">
         <is>
-          <t>A flame-scarred stray beast of the undercity, a charged rod.</t>
+          <t>A slow slick of marsh rot with an appetite, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -10003,7 +10003,7 @@
       </c>
       <c r="B125" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Shell Beast</t>
         </is>
       </c>
       <c r="C125" s="9" t="inlineStr">
@@ -10043,7 +10043,7 @@
       </c>
       <c r="L125" s="9" t="inlineStr">
         <is>
-          <t>A flame-scarred stray beast of the undercity, a charged rod.</t>
+          <t>A slab-shelled beast that shrugs off blows, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -10471,7 +10471,7 @@
       </c>
       <c r="B134" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C134" s="7" t="inlineStr">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="L134" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -10523,7 +10523,7 @@
       </c>
       <c r="B135" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>River Siren</t>
         </is>
       </c>
       <c r="C135" s="9" t="inlineStr">
@@ -10563,7 +10563,7 @@
       </c>
       <c r="L135" s="9" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a charged rod.</t>
+          <t>A pale water-spirit that sings the unwary under.</t>
         </is>
       </c>
     </row>
@@ -10835,7 +10835,7 @@
       </c>
       <c r="B141" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Sky Beast</t>
         </is>
       </c>
       <c r="C141" s="9" t="inlineStr">
@@ -10875,7 +10875,7 @@
       </c>
       <c r="L141" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A winged thing out of the reactor haze, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -10939,7 +10939,7 @@
       </c>
       <c r="B143" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C143" s="9" t="inlineStr">
@@ -10979,7 +10979,7 @@
       </c>
       <c r="L143" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -10991,7 +10991,7 @@
       </c>
       <c r="B144" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Swarm Machine</t>
         </is>
       </c>
       <c r="C144" s="7" t="inlineStr">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="L144" s="7" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a charged rod.</t>
+          <t>A cloud of tiny machines that moves and strikes as one.</t>
         </is>
       </c>
     </row>
@@ -11043,7 +11043,7 @@
       </c>
       <c r="B145" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>the Hollow</t>
         </is>
       </c>
       <c r="C145" s="9" t="inlineStr">
@@ -11083,7 +11083,7 @@
       </c>
       <c r="L145" s="9" t="inlineStr">
         <is>
-          <t>A night-black stray beast of the undercity, a charged rod.</t>
+          <t>A walking piece of absence, eating color and sound, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -11095,7 +11095,7 @@
       </c>
       <c r="B146" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Bone Caster</t>
         </is>
       </c>
       <c r="C146" s="7" t="inlineStr">
@@ -11135,7 +11135,7 @@
       </c>
       <c r="L146" s="7" t="inlineStr">
         <is>
-          <t>A night-black stray beast of the undercity, a charged rod.</t>
+          <t>A dead thing still working the dark, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -11147,7 +11147,7 @@
       </c>
       <c r="B147" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>the Hollow</t>
         </is>
       </c>
       <c r="C147" s="9" t="inlineStr">
@@ -11183,7 +11183,7 @@
       </c>
       <c r="L147" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A walking piece of absence, eating color and sound, bare claws.</t>
         </is>
       </c>
     </row>
@@ -11195,7 +11195,7 @@
       </c>
       <c r="B148" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>the Hollow</t>
         </is>
       </c>
       <c r="C148" s="7" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="L148" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A walking piece of absence, eating color and sound, bare claws.</t>
         </is>
       </c>
     </row>
@@ -11243,7 +11243,7 @@
       </c>
       <c r="B149" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>the Hollow</t>
         </is>
       </c>
       <c r="C149" s="9" t="inlineStr">
@@ -11283,7 +11283,7 @@
       </c>
       <c r="L149" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A walking piece of absence, eating color and sound, a long pike.</t>
         </is>
       </c>
     </row>
@@ -11295,7 +11295,7 @@
       </c>
       <c r="B150" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>the Hollow</t>
         </is>
       </c>
       <c r="C150" s="7" t="inlineStr">
@@ -11335,7 +11335,7 @@
       </c>
       <c r="L150" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A walking piece of absence, eating color and sound, a long pike.</t>
         </is>
       </c>
     </row>
@@ -11347,7 +11347,7 @@
       </c>
       <c r="B151" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>the Hollow</t>
         </is>
       </c>
       <c r="C151" s="9" t="inlineStr">
@@ -11387,7 +11387,7 @@
       </c>
       <c r="L151" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A walking piece of absence, eating color and sound, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -11399,7 +11399,7 @@
       </c>
       <c r="B152" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C152" s="7" t="inlineStr">
@@ -11439,7 +11439,7 @@
       </c>
       <c r="L152" s="7" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a long pike.</t>
+          <t>A frost-rimed beast of the undercity, a long pike.</t>
         </is>
       </c>
     </row>
@@ -12643,7 +12643,7 @@
       </c>
       <c r="B176" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Iron Crawler</t>
         </is>
       </c>
       <c r="C176" s="7" t="inlineStr">
@@ -12683,7 +12683,7 @@
       </c>
       <c r="L176" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A many-legged iron crawler that skitters along the walls, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -12747,7 +12747,7 @@
       </c>
       <c r="B178" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C178" s="7" t="inlineStr">
@@ -12787,7 +12787,7 @@
       </c>
       <c r="L178" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A beast of the undercity, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -13163,7 +13163,7 @@
       </c>
       <c r="B186" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Southbank Fighter</t>
         </is>
       </c>
       <c r="C186" s="7" t="inlineStr">
@@ -13203,7 +13203,7 @@
       </c>
       <c r="L186" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A Southbank outlaw, no flag in any file, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -13215,7 +13215,7 @@
       </c>
       <c r="B187" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Arc Machine</t>
         </is>
       </c>
       <c r="C187" s="9" t="inlineStr">
@@ -13255,7 +13255,7 @@
       </c>
       <c r="L187" s="9" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a compound bow.</t>
+          <t>A crackling Commission unit sheathed in live current, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -13267,7 +13267,7 @@
       </c>
       <c r="B188" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Southbank Fighter</t>
         </is>
       </c>
       <c r="C188" s="7" t="inlineStr">
@@ -13307,7 +13307,7 @@
       </c>
       <c r="L188" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A Southbank outlaw, no flag in any file, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -13319,7 +13319,7 @@
       </c>
       <c r="B189" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C189" s="9" t="inlineStr">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="L189" s="9" t="inlineStr">
         <is>
-          <t>A flame-scarred stray beast of the undercity, a charged rod.</t>
+          <t>A flame-scarred beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -13371,7 +13371,7 @@
       </c>
       <c r="B190" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C190" s="7" t="inlineStr">
@@ -13411,7 +13411,7 @@
       </c>
       <c r="L190" s="7" t="inlineStr">
         <is>
-          <t>A flame-scarred stray beast of the undercity, a long pike.</t>
+          <t>A flame-scarred beast of the undercity, a long pike.</t>
         </is>
       </c>
     </row>
@@ -13475,7 +13475,7 @@
       </c>
       <c r="B192" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C192" s="7" t="inlineStr">
@@ -13515,7 +13515,7 @@
       </c>
       <c r="L192" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A beast of the undercity, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -13527,7 +13527,7 @@
       </c>
       <c r="B193" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C193" s="9" t="inlineStr">
@@ -13567,7 +13567,7 @@
       </c>
       <c r="L193" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -13579,7 +13579,7 @@
       </c>
       <c r="B194" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Horned Beast</t>
         </is>
       </c>
       <c r="C194" s="7" t="inlineStr">
@@ -13619,7 +13619,7 @@
       </c>
       <c r="L194" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A heavy horned beast of the old wilds, a long pike.</t>
         </is>
       </c>
     </row>
@@ -13631,7 +13631,7 @@
       </c>
       <c r="B195" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Creeper</t>
         </is>
       </c>
       <c r="C195" s="9" t="inlineStr">
@@ -13671,7 +13671,7 @@
       </c>
       <c r="L195" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A low creeping horror that hugs the ground, a long pike.</t>
         </is>
       </c>
     </row>
@@ -13787,7 +13787,7 @@
       </c>
       <c r="B198" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Frost Beast</t>
         </is>
       </c>
       <c r="C198" s="7" t="inlineStr">
@@ -13827,7 +13827,7 @@
       </c>
       <c r="L198" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A hunched beast rimed in lake ice, breath like winter, a long pike.</t>
         </is>
       </c>
     </row>
@@ -13839,7 +13839,7 @@
       </c>
       <c r="B199" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C199" s="9" t="inlineStr">
@@ -13879,7 +13879,7 @@
       </c>
       <c r="L199" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -13995,7 +13995,7 @@
       </c>
       <c r="B202" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C202" s="7" t="inlineStr">
@@ -14035,7 +14035,7 @@
       </c>
       <c r="L202" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -14047,7 +14047,7 @@
       </c>
       <c r="B203" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C203" s="9" t="inlineStr">
@@ -14087,7 +14087,7 @@
       </c>
       <c r="L203" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A beast of the undercity, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -14099,7 +14099,7 @@
       </c>
       <c r="B204" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Sludge Beast</t>
         </is>
       </c>
       <c r="C204" s="7" t="inlineStr">
@@ -14139,7 +14139,7 @@
       </c>
       <c r="L204" s="7" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a charged rod.</t>
+          <t>A slow slick of marsh rot with an appetite, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -14151,7 +14151,7 @@
       </c>
       <c r="B205" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C205" s="9" t="inlineStr">
@@ -14191,7 +14191,7 @@
       </c>
       <c r="L205" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -14203,7 +14203,7 @@
       </c>
       <c r="B206" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C206" s="7" t="inlineStr">
@@ -14243,7 +14243,7 @@
       </c>
       <c r="L206" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -14463,7 +14463,7 @@
       </c>
       <c r="B211" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Blade Beast</t>
         </is>
       </c>
       <c r="C211" s="9" t="inlineStr">
@@ -14503,7 +14503,7 @@
       </c>
       <c r="L211" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A lean cutthroat shape all edges, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -14515,7 +14515,7 @@
       </c>
       <c r="B212" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Blade Beast</t>
         </is>
       </c>
       <c r="C212" s="7" t="inlineStr">
@@ -14555,7 +14555,7 @@
       </c>
       <c r="L212" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A lean cutthroat shape all edges, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -14567,7 +14567,7 @@
       </c>
       <c r="B213" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Blade Beast</t>
         </is>
       </c>
       <c r="C213" s="9" t="inlineStr">
@@ -14607,7 +14607,7 @@
       </c>
       <c r="L213" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a heavy blade.</t>
+          <t>A lean cutthroat shape all edges, a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -14671,7 +14671,7 @@
       </c>
       <c r="B215" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C215" s="9" t="inlineStr">
@@ -14711,7 +14711,7 @@
       </c>
       <c r="L215" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -14723,7 +14723,7 @@
       </c>
       <c r="B216" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C216" s="7" t="inlineStr">
@@ -14763,7 +14763,7 @@
       </c>
       <c r="L216" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -14827,7 +14827,7 @@
       </c>
       <c r="B218" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C218" s="7" t="inlineStr">
@@ -14867,7 +14867,7 @@
       </c>
       <c r="L218" s="7" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a charged rod.</t>
+          <t>A frost-rimed beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -14879,7 +14879,7 @@
       </c>
       <c r="B219" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C219" s="9" t="inlineStr">
@@ -14919,7 +14919,7 @@
       </c>
       <c r="L219" s="9" t="inlineStr">
         <is>
-          <t>A frost-rimed stray beast of the undercity, a charged rod.</t>
+          <t>A frost-rimed beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -14931,7 +14931,7 @@
       </c>
       <c r="B220" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C220" s="7" t="inlineStr">
@@ -14971,7 +14971,7 @@
       </c>
       <c r="L220" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -14983,7 +14983,7 @@
       </c>
       <c r="B221" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Fen Spirit</t>
         </is>
       </c>
       <c r="C221" s="9" t="inlineStr">
@@ -15023,7 +15023,7 @@
       </c>
       <c r="L221" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A marsh-wisp of the drowned undercity, a long pike.</t>
         </is>
       </c>
     </row>
@@ -15035,7 +15035,7 @@
       </c>
       <c r="B222" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Fen Spirit</t>
         </is>
       </c>
       <c r="C222" s="7" t="inlineStr">
@@ -15075,7 +15075,7 @@
       </c>
       <c r="L222" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A marsh-wisp of the drowned undercity, a long pike.</t>
         </is>
       </c>
     </row>
@@ -15087,7 +15087,7 @@
       </c>
       <c r="B223" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C223" s="9" t="inlineStr">
@@ -15123,7 +15123,7 @@
       </c>
       <c r="L223" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A beast of the undercity, bare claws.</t>
         </is>
       </c>
     </row>
@@ -15135,7 +15135,7 @@
       </c>
       <c r="B224" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C224" s="7" t="inlineStr">
@@ -15175,7 +15175,7 @@
       </c>
       <c r="L224" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -15395,7 +15395,7 @@
       </c>
       <c r="B229" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Enforcement Machine</t>
         </is>
       </c>
       <c r="C229" s="9" t="inlineStr">
@@ -15435,7 +15435,7 @@
       </c>
       <c r="L229" s="9" t="inlineStr">
         <is>
-          <t>A flame-scarred stray beast of the undercity, a heavy blade.</t>
+          <t>A heavy Commission war-machine, servos hissing, flame-scarred a heavy blade.</t>
         </is>
       </c>
     </row>
@@ -15447,7 +15447,7 @@
       </c>
       <c r="B230" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C230" s="7" t="inlineStr">
@@ -15487,7 +15487,7 @@
       </c>
       <c r="L230" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A beast of the undercity, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -15499,7 +15499,7 @@
       </c>
       <c r="B231" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Enforcement Machine</t>
         </is>
       </c>
       <c r="C231" s="9" t="inlineStr">
@@ -15539,7 +15539,7 @@
       </c>
       <c r="L231" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A heavy Commission war-machine, servos hissing, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -15551,7 +15551,7 @@
       </c>
       <c r="B232" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Horned Beast</t>
         </is>
       </c>
       <c r="C232" s="7" t="inlineStr">
@@ -15591,7 +15591,7 @@
       </c>
       <c r="L232" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a compound bow.</t>
+          <t>A heavy horned beast of the old wilds, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -15603,7 +15603,7 @@
       </c>
       <c r="B233" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Horned Beast</t>
         </is>
       </c>
       <c r="C233" s="9" t="inlineStr">
@@ -15643,7 +15643,7 @@
       </c>
       <c r="L233" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A heavy horned beast of the old wilds, a long pike.</t>
         </is>
       </c>
     </row>
@@ -15655,7 +15655,7 @@
       </c>
       <c r="B234" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Horned Beast</t>
         </is>
       </c>
       <c r="C234" s="7" t="inlineStr">
@@ -15695,7 +15695,7 @@
       </c>
       <c r="L234" s="7" t="inlineStr">
         <is>
-          <t>A storm-lit stray beast of the undercity, a charged rod.</t>
+          <t>A heavy horned beast of the old wilds, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -15811,7 +15811,7 @@
       </c>
       <c r="B237" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C237" s="9" t="inlineStr">
@@ -15851,7 +15851,7 @@
       </c>
       <c r="L237" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -15915,7 +15915,7 @@
       </c>
       <c r="B239" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Enforcement Machine</t>
         </is>
       </c>
       <c r="C239" s="9" t="inlineStr">
@@ -15955,7 +15955,7 @@
       </c>
       <c r="L239" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A heavy Commission war-machine, servos hissing, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -15967,7 +15967,7 @@
       </c>
       <c r="B240" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C240" s="7" t="inlineStr">
@@ -16007,7 +16007,7 @@
       </c>
       <c r="L240" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -16071,7 +16071,7 @@
       </c>
       <c r="B242" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C242" s="7" t="inlineStr">
@@ -16111,7 +16111,7 @@
       </c>
       <c r="L242" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a long pike.</t>
+          <t>A beast of the undercity, a long pike.</t>
         </is>
       </c>
     </row>
@@ -16123,7 +16123,7 @@
       </c>
       <c r="B243" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C243" s="9" t="inlineStr">
@@ -16163,7 +16163,7 @@
       </c>
       <c r="L243" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -16379,7 +16379,7 @@
       </c>
       <c r="B248" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C248" s="7" t="inlineStr">
@@ -16415,7 +16415,7 @@
       </c>
       <c r="L248" s="7" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A beast of the undercity, bare claws.</t>
         </is>
       </c>
     </row>
@@ -16427,7 +16427,7 @@
       </c>
       <c r="B249" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Fen Spirit</t>
         </is>
       </c>
       <c r="C249" s="9" t="inlineStr">
@@ -16463,7 +16463,7 @@
       </c>
       <c r="L249" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, bare claws.</t>
+          <t>A marsh-wisp of the drowned undercity, bare claws.</t>
         </is>
       </c>
     </row>
@@ -16475,7 +16475,7 @@
       </c>
       <c r="B250" s="6" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C250" s="7" t="inlineStr">
@@ -16515,7 +16515,7 @@
       </c>
       <c r="L250" s="7" t="inlineStr">
         <is>
-          <t>A flame-scarred stray beast of the undercity, a compound bow.</t>
+          <t>A flame-scarred beast of the undercity, a compound bow.</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="B251" s="8" t="inlineStr">
         <is>
-          <t>Stray Beast</t>
+          <t>Undercity Beast</t>
         </is>
       </c>
       <c r="C251" s="9" t="inlineStr">
@@ -16567,7 +16567,7 @@
       </c>
       <c r="L251" s="9" t="inlineStr">
         <is>
-          <t>A stray beast of the undercity, a charged rod.</t>
+          <t>A beast of the undercity, a charged rod.</t>
         </is>
       </c>
     </row>
@@ -22506,7 +22506,7 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>You don't even know us.</t>
+          <t>You don't even know us. I could be dangerous.</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -22516,7 +22516,7 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>You don't even know us.</t>
+          <t>You don't even know us. I could be dangerous.</t>
         </is>
       </c>
     </row>
@@ -23388,7 +23388,7 @@
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>SEE? It comes for everyone, planning lady.</t>
+          <t>SEE? Even you improvise now. There's hope for you yet, planning lady.</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
@@ -23398,7 +23398,7 @@
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>SEE? It comes for everyone, planning lady.</t>
+          <t>SEE? Even you improvise now. There's hope for you yet, planning lady.</t>
         </is>
       </c>
     </row>
@@ -25248,7 +25248,7 @@
       </c>
       <c r="D127" s="9" t="inlineStr">
         <is>
-          <t>At us?</t>
+          <t>At us? What did we do to rate our own monsters?</t>
         </is>
       </c>
       <c r="E127" s="8" t="inlineStr">
@@ -25258,7 +25258,7 @@
       </c>
       <c r="F127" s="9" t="inlineStr">
         <is>
-          <t>At us?</t>
+          <t>At us? What did we do to rate our own monsters?</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Outer Heaven reskin workbook
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Outer_Heaven_Reskin.xlsx
+++ b/Outer_Heaven_Reskin.xlsx
@@ -1865,8 +1865,8 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>The Commission answers the heist with its favorite hammer: Qin Ming, garrison champion, a man whose temper arrives before his orders do. The Wisdom Star baits him into the flood channels, beats him fair, and sends him home embarrassed.
-He gets there in time to watch the Commission burn his garrison for the crime of losing. They wrote him off as a failure, so they billed him the fire.
+          <t>The Commission answers the heist with its favorite hammer: Qin Ming, garrison champion, a man whose temper arrives before his orders do. The Wisdom Star baits his overcharged sentinels into the flood channels and shorts them out, one by one, until the champion is left commanding nothing but sparks.
+He gets home in time to watch the Commission burn that garrison for the crime of losing. They wrote him off as a failure, so they billed him the fire.
 He walks back to Outer Heaven carrying the ashes and his mace.</t>
         </is>
       </c>
@@ -1887,8 +1887,8 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Marshal Huyan Zhuo does not lose, and the Commission sends him to prove it. He comes down the lake road with armor columns and a career of medals, and Outer Heaven holds.
-Beaten fair, he asks for a rematch. Then, on his way out, he passes an enforcement squad burning a food line for the crime of feeding Deviants, and something in the marshal finishes changing sides before the rematch does.</t>
+          <t>Marshal Huyan Zhuo does not lose, and the Commission sends him to prove it. He comes down the lake road with armor columns and a career of medals, and the columns break against Outer Heaven's walls.
+Beaten for the first time in that career, he asks for a rematch. Then, on his way out, he passes an enforcement squad burning a food line for the crime of feeding Deviants, and something in the marshal finishes changing sides before the rematch does.</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -22390,7 +22390,7 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>You're the deviants from the bulletins. Did my own company predict me into this?</t>
+          <t>You're the deviants from the bulletins. Someone predicted me into ruin overnight. I intend to find out who.</t>
         </is>
       </c>
     </row>
@@ -22414,7 +22414,7 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Rich man, we can't afford your company. We got flagged the artisanal way.</t>
+          <t>Rich man, down here a prediction's a luxury. We got flagged the artisanal way.</t>
         </is>
       </c>
     </row>
@@ -22438,7 +22438,7 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Then stand still while I find out who could.</t>
+          <t>Then stand still while I find someone who could afford it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ch.26 banter: split the "crack" call into its own dialogue box; drop dashes
Yan Qing's line packed two ideas (why the Flawless One froze + strike now)
and the transition was unclear. Now two boxes: "It hesitated. It's never
seen us laugh." then "There's the crack. Hit it now." Also cleaned the
last 3 em dashes from the xlsx builder (docstring + workbook title).
No em dashes remain in any content source.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Outer_Heaven_Reskin.xlsx
+++ b/Outer_Heaven_Reskin.xlsx
@@ -503,7 +503,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HEAVEN'S MANDATE — Outer Heaven — Re-skin Mapping</t>
+          <t>HEAVEN'S MANDATE: Outer Heaven Re-skin Mapping</t>
         </is>
       </c>
     </row>
@@ -22015,7 +22015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F180"/>
+  <dimension ref="A1:F181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -24384,7 +24384,7 @@
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>Order's forged, broadcast is mine for ninety seconds. Run on go.</t>
+          <t>Forged order's on every screen in the plaza. Ninety seconds before they cut it. Run on go.</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -24394,7 +24394,7 @@
       </c>
       <c r="F93" s="9" t="inlineStr">
         <is>
-          <t>Order's forged, broadcast is mine for ninety seconds. Run on go.</t>
+          <t>Forged order's on every screen in the plaza. Ninety seconds before they cut it. Run on go.</t>
         </is>
       </c>
     </row>
@@ -24888,7 +24888,7 @@
       </c>
       <c r="D113" s="9" t="inlineStr">
         <is>
-          <t>It hesitated. Hit the flawless thing in the joke.</t>
+          <t>It hesitated. It's never seen us laugh.</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -24898,61 +24898,61 @@
       </c>
       <c r="F113" s="9" t="inlineStr">
         <is>
-          <t>It hesitated. Hit the flawless thing in the joke.</t>
+          <t>It hesitated. It's never seen us laugh.</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="7" t="n">
+      <c r="A114" s="7" t="inlineStr"/>
+      <c r="B114" s="6" t="inlineStr"/>
+      <c r="C114" s="7" t="inlineStr">
+        <is>
+          <t>the Wanderer</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="inlineStr">
+        <is>
+          <t>There's the crack. Hit it now.</t>
+        </is>
+      </c>
+      <c r="E114" s="6" t="inlineStr">
+        <is>
+          <t>THE WANDERER</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>There's the crack. Hit it now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B114" s="6" t="inlineStr">
+      <c r="B115" s="8" t="inlineStr">
         <is>
           <t>The Kitchen Goes Dark</t>
         </is>
       </c>
-      <c r="C114" s="7" t="inlineStr">
+      <c r="C115" s="9" t="inlineStr">
         <is>
           <t>the Tattooed Monk</t>
         </is>
       </c>
-      <c r="D114" s="7" t="inlineStr">
+      <c r="D115" s="9" t="inlineStr">
         <is>
           <t>The gate's still standing. She held it. So we hold the rest.</t>
         </is>
       </c>
-      <c r="E114" s="6" t="inlineStr">
+      <c r="E115" s="8" t="inlineStr">
         <is>
           <t>THE TATTOOED MONK</t>
         </is>
       </c>
-      <c r="F114" s="7" t="inlineStr">
+      <c r="F115" s="9" t="inlineStr">
         <is>
           <t>The gate's still standing. She held it. So we hold the rest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="9" t="inlineStr"/>
-      <c r="B115" s="8" t="inlineStr"/>
-      <c r="C115" s="9" t="inlineStr">
-        <is>
-          <t>Black Whirlwind</t>
-        </is>
-      </c>
-      <c r="D115" s="9" t="inlineStr">
-        <is>
-          <t>I'll cook tonight. She'd hate that. She'd yell.</t>
-        </is>
-      </c>
-      <c r="E115" s="8" t="inlineStr">
-        <is>
-          <t>BLACK WHIRLWIND</t>
-        </is>
-      </c>
-      <c r="F115" s="9" t="inlineStr">
-        <is>
-          <t>I'll cook tonight. She'd hate that. She'd yell.</t>
         </is>
       </c>
     </row>
@@ -24961,22 +24961,22 @@
       <c r="B116" s="6" t="inlineStr"/>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>the Tattooed Monk</t>
+          <t>Black Whirlwind</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>She'd love yelling. Cook badly, little brother. For her.</t>
+          <t>I'll cook tonight. She'd hate that. She'd yell.</t>
         </is>
       </c>
       <c r="E116" s="6" t="inlineStr">
         <is>
-          <t>THE TATTOOED MONK</t>
+          <t>BLACK WHIRLWIND</t>
         </is>
       </c>
       <c r="F116" s="7" t="inlineStr">
         <is>
-          <t>She'd love yelling. Cook badly, little brother. For her.</t>
+          <t>I'll cook tonight. She'd hate that. She'd yell.</t>
         </is>
       </c>
     </row>
@@ -24985,76 +24985,76 @@
       <c r="B117" s="8" t="inlineStr"/>
       <c r="C117" s="9" t="inlineStr">
         <is>
+          <t>the Tattooed Monk</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
+        <is>
+          <t>She'd love yelling. Cook badly, little brother. For her.</t>
+        </is>
+      </c>
+      <c r="E117" s="8" t="inlineStr">
+        <is>
+          <t>THE TATTOOED MONK</t>
+        </is>
+      </c>
+      <c r="F117" s="9" t="inlineStr">
+        <is>
+          <t>She'd love yelling. Cook badly, little brother. For her.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="7" t="inlineStr"/>
+      <c r="B118" s="6" t="inlineStr"/>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
           <t>Timely Rain</t>
         </is>
       </c>
-      <c r="D117" s="9" t="inlineStr">
+      <c r="D118" s="7" t="inlineStr">
         <is>
           <t>Line up. Children first, grief second. Her rules.</t>
         </is>
       </c>
-      <c r="E117" s="8" t="inlineStr">
+      <c r="E118" s="6" t="inlineStr">
         <is>
           <t>TIMELY RAIN</t>
         </is>
       </c>
-      <c r="F117" s="9" t="inlineStr">
+      <c r="F118" s="7" t="inlineStr">
         <is>
           <t>Line up. Children first, grief second. Her rules.</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="7" t="n">
+    <row r="119">
+      <c r="A119" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B118" s="6" t="inlineStr">
+      <c r="B119" s="8" t="inlineStr">
         <is>
           <t>What Grief Does</t>
         </is>
       </c>
-      <c r="C118" s="7" t="inlineStr">
+      <c r="C119" s="9" t="inlineStr">
         <is>
           <t>the Pilgrim</t>
         </is>
       </c>
-      <c r="D118" s="7" t="inlineStr">
+      <c r="D119" s="9" t="inlineStr">
         <is>
           <t>Don't say it. I know how this road ends. I walked it for my brother.</t>
         </is>
       </c>
-      <c r="E118" s="6" t="inlineStr">
+      <c r="E119" s="8" t="inlineStr">
         <is>
           <t>THE PILGRIM</t>
         </is>
       </c>
-      <c r="F118" s="7" t="inlineStr">
+      <c r="F119" s="9" t="inlineStr">
         <is>
           <t>Don't say it. I know how this road ends. I walked it for my brother.</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="9" t="inlineStr"/>
-      <c r="B119" s="8" t="inlineStr"/>
-      <c r="C119" s="9" t="inlineStr">
-        <is>
-          <t>the Skilled Doctor</t>
-        </is>
-      </c>
-      <c r="D119" s="9" t="inlineStr">
-        <is>
-          <t>I'm not saying anything. I'm setting your hand. It's broken.</t>
-        </is>
-      </c>
-      <c r="E119" s="8" t="inlineStr">
-        <is>
-          <t>THE SKILLED DOCTOR</t>
-        </is>
-      </c>
-      <c r="F119" s="9" t="inlineStr">
-        <is>
-          <t>I'm not saying anything. I'm setting your hand. It's broken.</t>
         </is>
       </c>
     </row>
@@ -25063,22 +25063,22 @@
       <c r="B120" s="6" t="inlineStr"/>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>the Pilgrim</t>
+          <t>the Skilled Doctor</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>It's fine.</t>
+          <t>I'm not saying anything. I'm setting your hand. It's broken.</t>
         </is>
       </c>
       <c r="E120" s="6" t="inlineStr">
         <is>
-          <t>THE PILGRIM</t>
+          <t>THE SKILLED DOCTOR</t>
         </is>
       </c>
       <c r="F120" s="7" t="inlineStr">
         <is>
-          <t>It's fine.</t>
+          <t>I'm not saying anything. I'm setting your hand. It's broken.</t>
         </is>
       </c>
     </row>
@@ -25087,76 +25087,76 @@
       <c r="B121" s="8" t="inlineStr"/>
       <c r="C121" s="9" t="inlineStr">
         <is>
+          <t>the Pilgrim</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>It's fine.</t>
+        </is>
+      </c>
+      <c r="E121" s="8" t="inlineStr">
+        <is>
+          <t>THE PILGRIM</t>
+        </is>
+      </c>
+      <c r="F121" s="9" t="inlineStr">
+        <is>
+          <t>It's fine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="7" t="inlineStr"/>
+      <c r="B122" s="6" t="inlineStr"/>
+      <c r="C122" s="7" t="inlineStr">
+        <is>
           <t>the Skilled Doctor</t>
         </is>
       </c>
-      <c r="D121" s="9" t="inlineStr">
+      <c r="D122" s="7" t="inlineStr">
         <is>
           <t>It's broken, and you're not. That's my report. We go home now.</t>
         </is>
       </c>
-      <c r="E121" s="8" t="inlineStr">
+      <c r="E122" s="6" t="inlineStr">
         <is>
           <t>THE SKILLED DOCTOR</t>
         </is>
       </c>
-      <c r="F121" s="9" t="inlineStr">
+      <c r="F122" s="7" t="inlineStr">
         <is>
           <t>It's broken, and you're not. That's my report. We go home now.</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="7" t="n">
+    <row r="123">
+      <c r="A123" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="B122" s="6" t="inlineStr">
+      <c r="B123" s="8" t="inlineStr">
         <is>
           <t>The Last Good Cop</t>
         </is>
       </c>
-      <c r="C122" s="7" t="inlineStr">
+      <c r="C123" s="9" t="inlineStr">
         <is>
           <t>Lord of the Beautiful Beard</t>
         </is>
       </c>
-      <c r="D122" s="7" t="inlineStr">
+      <c r="D123" s="9" t="inlineStr">
         <is>
           <t>You have the right to remain a monster. It waives the right.</t>
         </is>
       </c>
-      <c r="E122" s="6" t="inlineStr">
+      <c r="E123" s="8" t="inlineStr">
         <is>
           <t>LORD OF THE BEAUTIFUL BEARD</t>
         </is>
       </c>
-      <c r="F122" s="7" t="inlineStr">
+      <c r="F123" s="9" t="inlineStr">
         <is>
           <t>You have the right to remain a monster. It waives the right.</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="9" t="inlineStr"/>
-      <c r="B123" s="8" t="inlineStr"/>
-      <c r="C123" s="9" t="inlineStr">
-        <is>
-          <t>Black Whirlwind</t>
-        </is>
-      </c>
-      <c r="D123" s="9" t="inlineStr">
-        <is>
-          <t>Is he reading it its rights? It's a BEAST.</t>
-        </is>
-      </c>
-      <c r="E123" s="8" t="inlineStr">
-        <is>
-          <t>BLACK WHIRLWIND</t>
-        </is>
-      </c>
-      <c r="F123" s="9" t="inlineStr">
-        <is>
-          <t>Is he reading it its rights? It's a BEAST.</t>
         </is>
       </c>
     </row>
@@ -25165,22 +25165,22 @@
       <c r="B124" s="6" t="inlineStr"/>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>Lord of the Beautiful Beard</t>
+          <t>Black Whirlwind</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>Procedure survives employment, son.</t>
+          <t>Is he reading it its rights? It's a BEAST.</t>
         </is>
       </c>
       <c r="E124" s="6" t="inlineStr">
         <is>
-          <t>LORD OF THE BEAUTIFUL BEARD</t>
+          <t>BLACK WHIRLWIND</t>
         </is>
       </c>
       <c r="F124" s="7" t="inlineStr">
         <is>
-          <t>Procedure survives employment, son.</t>
+          <t>Is he reading it its rights? It's a BEAST.</t>
         </is>
       </c>
     </row>
@@ -25189,76 +25189,76 @@
       <c r="B125" s="8" t="inlineStr"/>
       <c r="C125" s="9" t="inlineStr">
         <is>
+          <t>Lord of the Beautiful Beard</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>Procedure survives employment, son.</t>
+        </is>
+      </c>
+      <c r="E125" s="8" t="inlineStr">
+        <is>
+          <t>LORD OF THE BEAUTIFUL BEARD</t>
+        </is>
+      </c>
+      <c r="F125" s="9" t="inlineStr">
+        <is>
+          <t>Procedure survives employment, son.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="7" t="inlineStr"/>
+      <c r="B126" s="6" t="inlineStr"/>
+      <c r="C126" s="7" t="inlineStr">
+        <is>
           <t>Ten Feet of Steel</t>
         </is>
       </c>
-      <c r="D125" s="9" t="inlineStr">
+      <c r="D126" s="7" t="inlineStr">
         <is>
           <t>Leave him be. The beard does the community outreach.</t>
         </is>
       </c>
-      <c r="E125" s="8" t="inlineStr">
+      <c r="E126" s="6" t="inlineStr">
         <is>
           <t>TEN FEET OF STEEL</t>
         </is>
       </c>
-      <c r="F125" s="9" t="inlineStr">
+      <c r="F126" s="7" t="inlineStr">
         <is>
           <t>Leave him be. The beard does the community outreach.</t>
         </is>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" s="7" t="n">
+    <row r="127">
+      <c r="A127" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B126" s="6" t="inlineStr">
+      <c r="B127" s="8" t="inlineStr">
         <is>
           <t>Folk Heroes</t>
         </is>
       </c>
-      <c r="C126" s="7" t="inlineStr">
+      <c r="C127" s="9" t="inlineStr">
         <is>
           <t>Two-Headed Snake</t>
         </is>
       </c>
-      <c r="D126" s="7" t="inlineStr">
+      <c r="D127" s="9" t="inlineStr">
         <is>
           <t>Beasts don't march in lines. Someone's herding them.</t>
         </is>
       </c>
-      <c r="E126" s="6" t="inlineStr">
+      <c r="E127" s="8" t="inlineStr">
         <is>
           <t>TWO-HEADED SNAKE</t>
         </is>
       </c>
-      <c r="F126" s="7" t="inlineStr">
+      <c r="F127" s="9" t="inlineStr">
         <is>
           <t>Beasts don't march in lines. Someone's herding them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="9" t="inlineStr"/>
-      <c r="B127" s="8" t="inlineStr"/>
-      <c r="C127" s="9" t="inlineStr">
-        <is>
-          <t>Nine Dragons</t>
-        </is>
-      </c>
-      <c r="D127" s="9" t="inlineStr">
-        <is>
-          <t>At us? What did we do to rate our own monsters?</t>
-        </is>
-      </c>
-      <c r="E127" s="8" t="inlineStr">
-        <is>
-          <t>NINE DRAGONS</t>
-        </is>
-      </c>
-      <c r="F127" s="9" t="inlineStr">
-        <is>
-          <t>At us? What did we do to rate our own monsters?</t>
         </is>
       </c>
     </row>
@@ -25267,22 +25267,22 @@
       <c r="B128" s="6" t="inlineStr"/>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>Two-Headed Snake</t>
+          <t>Nine Dragons</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>At whoever's being tested.</t>
+          <t>At us? What did we do to rate our own monsters?</t>
         </is>
       </c>
       <c r="E128" s="6" t="inlineStr">
         <is>
-          <t>TWO-HEADED SNAKE</t>
+          <t>NINE DRAGONS</t>
         </is>
       </c>
       <c r="F128" s="7" t="inlineStr">
         <is>
-          <t>At whoever's being tested.</t>
+          <t>At us? What did we do to rate our own monsters?</t>
         </is>
       </c>
     </row>
@@ -25291,76 +25291,76 @@
       <c r="B129" s="8" t="inlineStr"/>
       <c r="C129" s="9" t="inlineStr">
         <is>
+          <t>Two-Headed Snake</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>At whoever's being tested.</t>
+        </is>
+      </c>
+      <c r="E129" s="8" t="inlineStr">
+        <is>
+          <t>TWO-HEADED SNAKE</t>
+        </is>
+      </c>
+      <c r="F129" s="9" t="inlineStr">
+        <is>
+          <t>At whoever's being tested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="7" t="inlineStr"/>
+      <c r="B130" s="6" t="inlineStr"/>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
           <t>the Wisdom Star</t>
         </is>
       </c>
-      <c r="D129" s="9" t="inlineStr">
+      <c r="D130" s="7" t="inlineStr">
         <is>
           <t>Tested. There's that shape again.</t>
         </is>
       </c>
-      <c r="E129" s="8" t="inlineStr">
+      <c r="E130" s="6" t="inlineStr">
         <is>
           <t>THE WISDOM STAR</t>
         </is>
       </c>
-      <c r="F129" s="9" t="inlineStr">
+      <c r="F130" s="7" t="inlineStr">
         <is>
           <t>Tested. There's that shape again.</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="7" t="n">
+    <row r="131">
+      <c r="A131" s="9" t="n">
         <v>31</v>
       </c>
-      <c r="B130" s="6" t="inlineStr">
+      <c r="B131" s="8" t="inlineStr">
         <is>
           <t>Beast Country</t>
         </is>
       </c>
-      <c r="C130" s="7" t="inlineStr">
+      <c r="C131" s="9" t="inlineStr">
         <is>
           <t>Twin-Tailed Scorpion</t>
         </is>
       </c>
-      <c r="D130" s="7" t="inlineStr">
+      <c r="D131" s="9" t="inlineStr">
         <is>
           <t>...and THAT is why you flank a horn-king left.</t>
         </is>
       </c>
-      <c r="E130" s="6" t="inlineStr">
+      <c r="E131" s="8" t="inlineStr">
         <is>
           <t>TWIN-TAILED SCORPION</t>
         </is>
       </c>
-      <c r="F130" s="7" t="inlineStr">
+      <c r="F131" s="9" t="inlineStr">
         <is>
           <t>...and THAT is why you flank a horn-king left.</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="9" t="inlineStr"/>
-      <c r="B131" s="8" t="inlineStr"/>
-      <c r="C131" s="9" t="inlineStr">
-        <is>
-          <t>Two-Headed Snake</t>
-        </is>
-      </c>
-      <c r="D131" s="9" t="inlineStr">
-        <is>
-          <t>Started that sentence Tuesday.</t>
-        </is>
-      </c>
-      <c r="E131" s="8" t="inlineStr">
-        <is>
-          <t>TWO-HEADED SNAKE</t>
-        </is>
-      </c>
-      <c r="F131" s="9" t="inlineStr">
-        <is>
-          <t>Started that sentence Tuesday.</t>
         </is>
       </c>
     </row>
@@ -25369,22 +25369,22 @@
       <c r="B132" s="6" t="inlineStr"/>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>Twin-Tailed Scorpion</t>
+          <t>Two-Headed Snake</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>Finished it, didn't I?</t>
+          <t>Started that sentence Tuesday.</t>
         </is>
       </c>
       <c r="E132" s="6" t="inlineStr">
         <is>
-          <t>TWIN-TAILED SCORPION</t>
+          <t>TWO-HEADED SNAKE</t>
         </is>
       </c>
       <c r="F132" s="7" t="inlineStr">
         <is>
-          <t>Finished it, didn't I?</t>
+          <t>Started that sentence Tuesday.</t>
         </is>
       </c>
     </row>
@@ -25393,76 +25393,76 @@
       <c r="B133" s="8" t="inlineStr"/>
       <c r="C133" s="9" t="inlineStr">
         <is>
+          <t>Twin-Tailed Scorpion</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>Finished it, didn't I?</t>
+        </is>
+      </c>
+      <c r="E133" s="8" t="inlineStr">
+        <is>
+          <t>TWIN-TAILED SCORPION</t>
+        </is>
+      </c>
+      <c r="F133" s="9" t="inlineStr">
+        <is>
+          <t>Finished it, didn't I?</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="7" t="inlineStr"/>
+      <c r="B134" s="6" t="inlineStr"/>
+      <c r="C134" s="7" t="inlineStr">
+        <is>
           <t>the Skilled Doctor</t>
         </is>
       </c>
-      <c r="D133" s="9" t="inlineStr">
+      <c r="D134" s="7" t="inlineStr">
         <is>
           <t>There are two of them now. Archers bunk separately. Hunters bunk outside.</t>
         </is>
       </c>
-      <c r="E133" s="8" t="inlineStr">
+      <c r="E134" s="6" t="inlineStr">
         <is>
           <t>THE SKILLED DOCTOR</t>
         </is>
       </c>
-      <c r="F133" s="9" t="inlineStr">
+      <c r="F134" s="7" t="inlineStr">
         <is>
           <t>There are two of them now. Archers bunk separately. Hunters bunk outside.</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="7" t="n">
+    <row r="135">
+      <c r="A135" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="B134" s="6" t="inlineStr">
+      <c r="B135" s="8" t="inlineStr">
         <is>
           <t>The Southbank</t>
         </is>
       </c>
-      <c r="C134" s="7" t="inlineStr">
+      <c r="C135" s="9" t="inlineStr">
         <is>
           <t>the Witch</t>
         </is>
       </c>
-      <c r="D134" s="7" t="inlineStr">
+      <c r="D135" s="9" t="inlineStr">
         <is>
           <t>House rules: eat what I serve, start nothing, tip well. You'd all sell beautifully.</t>
         </is>
       </c>
-      <c r="E134" s="6" t="inlineStr">
+      <c r="E135" s="8" t="inlineStr">
         <is>
           <t>THE WITCH</t>
         </is>
       </c>
-      <c r="F134" s="7" t="inlineStr">
+      <c r="F135" s="9" t="inlineStr">
         <is>
           <t>House rules: eat what I serve, start nothing, tip well. You'd all sell beautifully.</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="9" t="inlineStr"/>
-      <c r="B135" s="8" t="inlineStr"/>
-      <c r="C135" s="9" t="inlineStr">
-        <is>
-          <t>the Wanderer</t>
-        </is>
-      </c>
-      <c r="D135" s="9" t="inlineStr">
-        <is>
-          <t>Was that a threat or a compliment?</t>
-        </is>
-      </c>
-      <c r="E135" s="8" t="inlineStr">
-        <is>
-          <t>THE WANDERER</t>
-        </is>
-      </c>
-      <c r="F135" s="9" t="inlineStr">
-        <is>
-          <t>Was that a threat or a compliment?</t>
         </is>
       </c>
     </row>
@@ -25471,22 +25471,22 @@
       <c r="B136" s="6" t="inlineStr"/>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>the Witch</t>
+          <t>the Wanderer</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>It's a menu.</t>
+          <t>Was that a threat or a compliment?</t>
         </is>
       </c>
       <c r="E136" s="6" t="inlineStr">
         <is>
-          <t>THE WITCH</t>
+          <t>THE WANDERER</t>
         </is>
       </c>
       <c r="F136" s="7" t="inlineStr">
         <is>
-          <t>It's a menu.</t>
+          <t>Was that a threat or a compliment?</t>
         </is>
       </c>
     </row>
@@ -25495,76 +25495,76 @@
       <c r="B137" s="8" t="inlineStr"/>
       <c r="C137" s="9" t="inlineStr">
         <is>
+          <t>the Witch</t>
+        </is>
+      </c>
+      <c r="D137" s="9" t="inlineStr">
+        <is>
+          <t>It's a menu.</t>
+        </is>
+      </c>
+      <c r="E137" s="8" t="inlineStr">
+        <is>
+          <t>THE WITCH</t>
+        </is>
+      </c>
+      <c r="F137" s="9" t="inlineStr">
+        <is>
+          <t>It's a menu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="7" t="inlineStr"/>
+      <c r="B138" s="6" t="inlineStr"/>
+      <c r="C138" s="7" t="inlineStr">
+        <is>
           <t>Red-Haired Devil</t>
         </is>
       </c>
-      <c r="D137" s="9" t="inlineStr">
+      <c r="D138" s="7" t="inlineStr">
         <is>
           <t>I like her. I'm terrified. Both.</t>
         </is>
       </c>
-      <c r="E137" s="8" t="inlineStr">
+      <c r="E138" s="6" t="inlineStr">
         <is>
           <t>RED-HAIRED DEVIL</t>
         </is>
       </c>
-      <c r="F137" s="9" t="inlineStr">
+      <c r="F138" s="7" t="inlineStr">
         <is>
           <t>I like her. I'm terrified. Both.</t>
         </is>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" s="7" t="n">
+    <row r="139">
+      <c r="A139" s="9" t="n">
         <v>33</v>
       </c>
-      <c r="B138" s="6" t="inlineStr">
+      <c r="B139" s="8" t="inlineStr">
         <is>
           <t>Written Into War</t>
         </is>
       </c>
-      <c r="C138" s="7" t="inlineStr">
+      <c r="C139" s="9" t="inlineStr">
         <is>
           <t>the Witch</t>
         </is>
       </c>
-      <c r="D138" s="7" t="inlineStr">
+      <c r="D139" s="9" t="inlineStr">
         <is>
           <t>My inn. Thirty years of soup. Someone burned it in twenty minutes.</t>
         </is>
       </c>
-      <c r="E138" s="6" t="inlineStr">
+      <c r="E139" s="8" t="inlineStr">
         <is>
           <t>THE WITCH</t>
         </is>
       </c>
-      <c r="F138" s="7" t="inlineStr">
+      <c r="F139" s="9" t="inlineStr">
         <is>
           <t>My inn. Thirty years of soup. Someone burned it in twenty minutes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="9" t="inlineStr"/>
-      <c r="B139" s="8" t="inlineStr"/>
-      <c r="C139" s="9" t="inlineStr">
-        <is>
-          <t>the Wisdom Star</t>
-        </is>
-      </c>
-      <c r="D139" s="9" t="inlineStr">
-        <is>
-          <t>The knots are wrong. Southbank hands don't tie like that. This was authored.</t>
-        </is>
-      </c>
-      <c r="E139" s="8" t="inlineStr">
-        <is>
-          <t>THE WISDOM STAR</t>
-        </is>
-      </c>
-      <c r="F139" s="9" t="inlineStr">
-        <is>
-          <t>The knots are wrong. Southbank hands don't tie like that. This was authored.</t>
         </is>
       </c>
     </row>
@@ -25573,22 +25573,22 @@
       <c r="B140" s="6" t="inlineStr"/>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>Fiery Thunderbolt</t>
+          <t>the Wisdom Star</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>Then point me at the author.</t>
+          <t>The knots are wrong. Southbank hands don't tie like that. This was authored.</t>
         </is>
       </c>
       <c r="E140" s="6" t="inlineStr">
         <is>
-          <t>FIERY THUNDERBOLT</t>
+          <t>THE WISDOM STAR</t>
         </is>
       </c>
       <c r="F140" s="7" t="inlineStr">
         <is>
-          <t>Then point me at the author.</t>
+          <t>The knots are wrong. Southbank hands don't tie like that. This was authored.</t>
         </is>
       </c>
     </row>
@@ -25597,76 +25597,76 @@
       <c r="B141" s="8" t="inlineStr"/>
       <c r="C141" s="9" t="inlineStr">
         <is>
+          <t>Fiery Thunderbolt</t>
+        </is>
+      </c>
+      <c r="D141" s="9" t="inlineStr">
+        <is>
+          <t>Then point me at the author.</t>
+        </is>
+      </c>
+      <c r="E141" s="8" t="inlineStr">
+        <is>
+          <t>FIERY THUNDERBOLT</t>
+        </is>
+      </c>
+      <c r="F141" s="9" t="inlineStr">
+        <is>
+          <t>Then point me at the author.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="7" t="inlineStr"/>
+      <c r="B142" s="6" t="inlineStr"/>
+      <c r="C142" s="7" t="inlineStr">
+        <is>
           <t>the Wisdom Star</t>
         </is>
       </c>
-      <c r="D141" s="9" t="inlineStr">
+      <c r="D142" s="7" t="inlineStr">
         <is>
           <t>That's the problem. There isn't one. Anywhere.</t>
         </is>
       </c>
-      <c r="E141" s="8" t="inlineStr">
+      <c r="E142" s="6" t="inlineStr">
         <is>
           <t>THE WISDOM STAR</t>
         </is>
       </c>
-      <c r="F141" s="9" t="inlineStr">
+      <c r="F142" s="7" t="inlineStr">
         <is>
           <t>That's the problem. There isn't one. Anywhere.</t>
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="7" t="n">
+    <row r="143">
+      <c r="A143" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="B142" s="6" t="inlineStr">
+      <c r="B143" s="8" t="inlineStr">
         <is>
           <t>The Offer</t>
         </is>
       </c>
-      <c r="C142" s="7" t="inlineStr">
+      <c r="C143" s="9" t="inlineStr">
         <is>
           <t>Gold Lancer</t>
         </is>
       </c>
-      <c r="D142" s="7" t="inlineStr">
+      <c r="D143" s="9" t="inlineStr">
         <is>
           <t>Feet wider. Commission armor opens at the collar, like a lie.</t>
         </is>
       </c>
-      <c r="E142" s="6" t="inlineStr">
+      <c r="E143" s="8" t="inlineStr">
         <is>
           <t>GOLD LANCER</t>
         </is>
       </c>
-      <c r="F142" s="7" t="inlineStr">
+      <c r="F143" s="9" t="inlineStr">
         <is>
           <t>Feet wider. Commission armor opens at the collar, like a lie.</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="9" t="inlineStr"/>
-      <c r="B143" s="8" t="inlineStr"/>
-      <c r="C143" s="9" t="inlineStr">
-        <is>
-          <t>Twin Rods</t>
-        </is>
-      </c>
-      <c r="D143" s="9" t="inlineStr">
-        <is>
-          <t>I wore that armor, lancer.</t>
-        </is>
-      </c>
-      <c r="E143" s="8" t="inlineStr">
-        <is>
-          <t>TWIN RODS</t>
-        </is>
-      </c>
-      <c r="F143" s="9" t="inlineStr">
-        <is>
-          <t>I wore that armor, lancer.</t>
         </is>
       </c>
     </row>
@@ -25675,22 +25675,22 @@
       <c r="B144" s="6" t="inlineStr"/>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>Gold Lancer</t>
+          <t>Twin Rods</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>Then you know where it lies.</t>
+          <t>I wore that armor, lancer.</t>
         </is>
       </c>
       <c r="E144" s="6" t="inlineStr">
         <is>
-          <t>GOLD LANCER</t>
+          <t>TWIN RODS</t>
         </is>
       </c>
       <c r="F144" s="7" t="inlineStr">
         <is>
-          <t>Then you know where it lies.</t>
+          <t>I wore that armor, lancer.</t>
         </is>
       </c>
     </row>
@@ -25699,76 +25699,76 @@
       <c r="B145" s="8" t="inlineStr"/>
       <c r="C145" s="9" t="inlineStr">
         <is>
+          <t>Gold Lancer</t>
+        </is>
+      </c>
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>Then you know where it lies.</t>
+        </is>
+      </c>
+      <c r="E145" s="8" t="inlineStr">
+        <is>
+          <t>GOLD LANCER</t>
+        </is>
+      </c>
+      <c r="F145" s="9" t="inlineStr">
+        <is>
+          <t>Then you know where it lies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="7" t="inlineStr"/>
+      <c r="B146" s="6" t="inlineStr"/>
+      <c r="C146" s="7" t="inlineStr">
+        <is>
           <t>Timely Rain</t>
         </is>
       </c>
-      <c r="D145" s="9" t="inlineStr">
+      <c r="D146" s="7" t="inlineStr">
         <is>
           <t>Rest well tonight. Tomorrow we decide who we are.</t>
         </is>
       </c>
-      <c r="E145" s="8" t="inlineStr">
+      <c r="E146" s="6" t="inlineStr">
         <is>
           <t>TIMELY RAIN</t>
         </is>
       </c>
-      <c r="F145" s="9" t="inlineStr">
+      <c r="F146" s="7" t="inlineStr">
         <is>
           <t>Rest well tonight. Tomorrow we decide who we are.</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="7" t="n">
+    <row r="147">
+      <c r="A147" s="9" t="n">
         <v>35</v>
       </c>
-      <c r="B146" s="6" t="inlineStr">
+      <c r="B147" s="8" t="inlineStr">
         <is>
           <t>The Vote</t>
         </is>
       </c>
-      <c r="C146" s="7" t="inlineStr">
+      <c r="C147" s="9" t="inlineStr">
         <is>
           <t>Black Whirlwind</t>
         </is>
       </c>
-      <c r="D146" s="7" t="inlineStr">
+      <c r="D147" s="9" t="inlineStr">
         <is>
           <t>Badges. BADGES. We're the ones they badge AGAINST.</t>
         </is>
       </c>
-      <c r="E146" s="6" t="inlineStr">
+      <c r="E147" s="8" t="inlineStr">
         <is>
           <t>BLACK WHIRLWIND</t>
         </is>
       </c>
-      <c r="F146" s="7" t="inlineStr">
+      <c r="F147" s="9" t="inlineStr">
         <is>
           <t>Badges. BADGES. We're the ones they badge AGAINST.</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="9" t="inlineStr"/>
-      <c r="B147" s="8" t="inlineStr"/>
-      <c r="C147" s="9" t="inlineStr">
-        <is>
-          <t>Timely Rain</t>
-        </is>
-      </c>
-      <c r="D147" s="9" t="inlineStr">
-        <is>
-          <t>And now they can't. Brother, I am trying to buy you a future.</t>
-        </is>
-      </c>
-      <c r="E147" s="8" t="inlineStr">
-        <is>
-          <t>TIMELY RAIN</t>
-        </is>
-      </c>
-      <c r="F147" s="9" t="inlineStr">
-        <is>
-          <t>And now they can't. Brother, I am trying to buy you a future.</t>
         </is>
       </c>
     </row>
@@ -25777,22 +25777,22 @@
       <c r="B148" s="6" t="inlineStr"/>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>Black Whirlwind</t>
+          <t>Timely Rain</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>Buy back the old one. I liked knowing who I was.</t>
+          <t>And now they can't. Brother, I am trying to buy you a future.</t>
         </is>
       </c>
       <c r="E148" s="6" t="inlineStr">
         <is>
-          <t>BLACK WHIRLWIND</t>
+          <t>TIMELY RAIN</t>
         </is>
       </c>
       <c r="F148" s="7" t="inlineStr">
         <is>
-          <t>Buy back the old one. I liked knowing who I was.</t>
+          <t>And now they can't. Brother, I am trying to buy you a future.</t>
         </is>
       </c>
     </row>
@@ -25801,76 +25801,76 @@
       <c r="B149" s="8" t="inlineStr"/>
       <c r="C149" s="9" t="inlineStr">
         <is>
+          <t>Black Whirlwind</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>Buy back the old one. I liked knowing who I was.</t>
+        </is>
+      </c>
+      <c r="E149" s="8" t="inlineStr">
+        <is>
+          <t>BLACK WHIRLWIND</t>
+        </is>
+      </c>
+      <c r="F149" s="9" t="inlineStr">
+        <is>
+          <t>Buy back the old one. I liked knowing who I was.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="7" t="inlineStr"/>
+      <c r="B150" s="6" t="inlineStr"/>
+      <c r="C150" s="7" t="inlineStr">
+        <is>
           <t>Panther Head</t>
         </is>
       </c>
-      <c r="D149" s="9" t="inlineStr">
+      <c r="D150" s="7" t="inlineStr">
         <is>
           <t>Wear it or don't. Tomorrow we march either way. Sleep.</t>
         </is>
       </c>
-      <c r="E149" s="8" t="inlineStr">
+      <c r="E150" s="6" t="inlineStr">
         <is>
           <t>PANTHER HEAD</t>
         </is>
       </c>
-      <c r="F149" s="9" t="inlineStr">
+      <c r="F150" s="7" t="inlineStr">
         <is>
           <t>Wear it or don't. Tomorrow we march either way. Sleep.</t>
         </is>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="7" t="n">
+    <row r="151">
+      <c r="A151" s="9" t="n">
         <v>36</v>
       </c>
-      <c r="B150" s="6" t="inlineStr">
+      <c r="B151" s="8" t="inlineStr">
         <is>
           <t>The War We Wanted</t>
         </is>
       </c>
-      <c r="C150" s="7" t="inlineStr">
+      <c r="C151" s="9" t="inlineStr">
         <is>
           <t>Fiery Thunderbolt</t>
         </is>
       </c>
-      <c r="D150" s="7" t="inlineStr">
+      <c r="D151" s="9" t="inlineStr">
         <is>
           <t>A bridge. Good. Bridges are honest work.</t>
         </is>
       </c>
-      <c r="E150" s="6" t="inlineStr">
+      <c r="E151" s="8" t="inlineStr">
         <is>
           <t>FIERY THUNDERBOLT</t>
         </is>
       </c>
-      <c r="F150" s="7" t="inlineStr">
+      <c r="F151" s="9" t="inlineStr">
         <is>
           <t>A bridge. Good. Bridges are honest work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="9" t="inlineStr"/>
-      <c r="B151" s="8" t="inlineStr"/>
-      <c r="C151" s="9" t="inlineStr">
-        <is>
-          <t>the Wisdom Star</t>
-        </is>
-      </c>
-      <c r="D151" s="9" t="inlineStr">
-        <is>
-          <t>Hold it four minutes, then fall back. Four. Minutes.</t>
-        </is>
-      </c>
-      <c r="E151" s="8" t="inlineStr">
-        <is>
-          <t>THE WISDOM STAR</t>
-        </is>
-      </c>
-      <c r="F151" s="9" t="inlineStr">
-        <is>
-          <t>Hold it four minutes, then fall back. Four. Minutes.</t>
         </is>
       </c>
     </row>
@@ -25879,22 +25879,22 @@
       <c r="B152" s="6" t="inlineStr"/>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>Fiery Thunderbolt</t>
+          <t>the Wisdom Star</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>Four minutes. Then I apologize to whatever's left standing.</t>
+          <t>Hold it four minutes, then fall back. Four. Minutes.</t>
         </is>
       </c>
       <c r="E152" s="6" t="inlineStr">
         <is>
-          <t>FIERY THUNDERBOLT</t>
+          <t>THE WISDOM STAR</t>
         </is>
       </c>
       <c r="F152" s="7" t="inlineStr">
         <is>
-          <t>Four minutes. Then I apologize to whatever's left standing.</t>
+          <t>Hold it four minutes, then fall back. Four. Minutes.</t>
         </is>
       </c>
     </row>
@@ -25903,76 +25903,76 @@
       <c r="B153" s="8" t="inlineStr"/>
       <c r="C153" s="9" t="inlineStr">
         <is>
+          <t>Fiery Thunderbolt</t>
+        </is>
+      </c>
+      <c r="D153" s="9" t="inlineStr">
+        <is>
+          <t>Four minutes. Then I apologize to whatever's left standing.</t>
+        </is>
+      </c>
+      <c r="E153" s="8" t="inlineStr">
+        <is>
+          <t>FIERY THUNDERBOLT</t>
+        </is>
+      </c>
+      <c r="F153" s="9" t="inlineStr">
+        <is>
+          <t>Four minutes. Then I apologize to whatever's left standing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="7" t="inlineStr"/>
+      <c r="B154" s="6" t="inlineStr"/>
+      <c r="C154" s="7" t="inlineStr">
+        <is>
           <t>the Witch</t>
         </is>
       </c>
-      <c r="D153" s="9" t="inlineStr">
+      <c r="D154" s="7" t="inlineStr">
         <is>
           <t>Come back hungry, thunder-man. I'm cooking for the loud ones tonight.</t>
         </is>
       </c>
-      <c r="E153" s="8" t="inlineStr">
+      <c r="E154" s="6" t="inlineStr">
         <is>
           <t>THE WITCH</t>
         </is>
       </c>
-      <c r="F153" s="9" t="inlineStr">
+      <c r="F154" s="7" t="inlineStr">
         <is>
           <t>Come back hungry, thunder-man. I'm cooking for the loud ones tonight.</t>
         </is>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="7" t="n">
+    <row r="155">
+      <c r="A155" s="9" t="n">
         <v>37</v>
       </c>
-      <c r="B154" s="6" t="inlineStr">
+      <c r="B155" s="8" t="inlineStr">
         <is>
           <t>The Water Gate</t>
         </is>
       </c>
-      <c r="C154" s="7" t="inlineStr">
+      <c r="C155" s="9" t="inlineStr">
         <is>
           <t>White Streak in the Waves</t>
         </is>
       </c>
-      <c r="D154" s="7" t="inlineStr">
+      <c r="D155" s="9" t="inlineStr">
         <is>
           <t>The gate holds if someone holds it. Water's honest. It should be me.</t>
         </is>
       </c>
-      <c r="E154" s="6" t="inlineStr">
+      <c r="E155" s="8" t="inlineStr">
         <is>
           <t>WHITE STREAK IN THE WAVES</t>
         </is>
       </c>
-      <c r="F154" s="7" t="inlineStr">
+      <c r="F155" s="9" t="inlineStr">
         <is>
           <t>The gate holds if someone holds it. Water's honest. It should be me.</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="9" t="inlineStr"/>
-      <c r="B155" s="8" t="inlineStr"/>
-      <c r="C155" s="9" t="inlineStr">
-        <is>
-          <t>Black Whirlwind</t>
-        </is>
-      </c>
-      <c r="D155" s="9" t="inlineStr">
-        <is>
-          <t>Then I hold YOU. That's the deal, fish. Land holds water.</t>
-        </is>
-      </c>
-      <c r="E155" s="8" t="inlineStr">
-        <is>
-          <t>BLACK WHIRLWIND</t>
-        </is>
-      </c>
-      <c r="F155" s="9" t="inlineStr">
-        <is>
-          <t>Then I hold YOU. That's the deal, fish. Land holds water.</t>
         </is>
       </c>
     </row>
@@ -25981,22 +25981,22 @@
       <c r="B156" s="6" t="inlineStr"/>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>White Streak in the Waves</t>
+          <t>Black Whirlwind</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>Not this time, land. Come in when it's over. The water will remember you.</t>
+          <t>Then I hold YOU. That's the deal, fish. Land holds water.</t>
         </is>
       </c>
       <c r="E156" s="6" t="inlineStr">
         <is>
-          <t>WHITE STREAK IN THE WAVES</t>
+          <t>BLACK WHIRLWIND</t>
         </is>
       </c>
       <c r="F156" s="7" t="inlineStr">
         <is>
-          <t>Not this time, land. Come in when it's over. The water will remember you.</t>
+          <t>Then I hold YOU. That's the deal, fish. Land holds water.</t>
         </is>
       </c>
     </row>
@@ -26005,76 +26005,76 @@
       <c r="B157" s="8" t="inlineStr"/>
       <c r="C157" s="9" t="inlineStr">
         <is>
+          <t>White Streak in the Waves</t>
+        </is>
+      </c>
+      <c r="D157" s="9" t="inlineStr">
+        <is>
+          <t>Not this time, land. Come in when it's over. The water will remember you.</t>
+        </is>
+      </c>
+      <c r="E157" s="8" t="inlineStr">
+        <is>
+          <t>WHITE STREAK IN THE WAVES</t>
+        </is>
+      </c>
+      <c r="F157" s="9" t="inlineStr">
+        <is>
+          <t>Not this time, land. Come in when it's over. The water will remember you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="7" t="inlineStr"/>
+      <c r="B158" s="6" t="inlineStr"/>
+      <c r="C158" s="7" t="inlineStr">
+        <is>
           <t>Red-Haired Devil</t>
         </is>
       </c>
-      <c r="D157" s="9" t="inlineStr">
+      <c r="D158" s="7" t="inlineStr">
         <is>
           <t>No plans, no speeches. See you all at the noodles.</t>
         </is>
       </c>
-      <c r="E157" s="8" t="inlineStr">
+      <c r="E158" s="6" t="inlineStr">
         <is>
           <t>RED-HAIRED DEVIL</t>
         </is>
       </c>
-      <c r="F157" s="9" t="inlineStr">
+      <c r="F158" s="7" t="inlineStr">
         <is>
           <t>No plans, no speeches. See you all at the noodles.</t>
         </is>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" s="7" t="n">
+    <row r="159">
+      <c r="A159" s="9" t="n">
         <v>38</v>
       </c>
-      <c r="B158" s="6" t="inlineStr">
+      <c r="B159" s="8" t="inlineStr">
         <is>
           <t>Counting</t>
         </is>
       </c>
-      <c r="C158" s="7" t="inlineStr">
+      <c r="C159" s="9" t="inlineStr">
         <is>
           <t>the Wisdom Star</t>
         </is>
       </c>
-      <c r="D158" s="7" t="inlineStr">
+      <c r="D159" s="9" t="inlineStr">
         <is>
           <t>I need everyone to hear this sober. Our whole war fits one curve.</t>
         </is>
       </c>
-      <c r="E158" s="6" t="inlineStr">
+      <c r="E159" s="8" t="inlineStr">
         <is>
           <t>THE WISDOM STAR</t>
         </is>
       </c>
-      <c r="F158" s="7" t="inlineStr">
+      <c r="F159" s="9" t="inlineStr">
         <is>
           <t>I need everyone to hear this sober. Our whole war fits one curve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="9" t="inlineStr"/>
-      <c r="B159" s="8" t="inlineStr"/>
-      <c r="C159" s="9" t="inlineStr">
-        <is>
-          <t>Panther Head</t>
-        </is>
-      </c>
-      <c r="D159" s="9" t="inlineStr">
-        <is>
-          <t>Meaning what?</t>
-        </is>
-      </c>
-      <c r="E159" s="8" t="inlineStr">
-        <is>
-          <t>PANTHER HEAD</t>
-        </is>
-      </c>
-      <c r="F159" s="9" t="inlineStr">
-        <is>
-          <t>Meaning what?</t>
         </is>
       </c>
     </row>
@@ -26083,22 +26083,22 @@
       <c r="B160" s="6" t="inlineStr"/>
       <c r="C160" s="7" t="inlineStr">
         <is>
-          <t>the Wisdom Star</t>
+          <t>Panther Head</t>
         </is>
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>Meaning somebody graded it. I found the rubric. It's older than the city.</t>
+          <t>Meaning what?</t>
         </is>
       </c>
       <c r="E160" s="6" t="inlineStr">
         <is>
-          <t>THE WISDOM STAR</t>
+          <t>PANTHER HEAD</t>
         </is>
       </c>
       <c r="F160" s="7" t="inlineStr">
         <is>
-          <t>Meaning somebody graded it. I found the rubric. It's older than the city.</t>
+          <t>Meaning what?</t>
         </is>
       </c>
     </row>
@@ -26107,76 +26107,76 @@
       <c r="B161" s="8" t="inlineStr"/>
       <c r="C161" s="9" t="inlineStr">
         <is>
+          <t>the Wisdom Star</t>
+        </is>
+      </c>
+      <c r="D161" s="9" t="inlineStr">
+        <is>
+          <t>Meaning somebody graded it. I found the rubric. It's older than the city.</t>
+        </is>
+      </c>
+      <c r="E161" s="8" t="inlineStr">
+        <is>
+          <t>THE WISDOM STAR</t>
+        </is>
+      </c>
+      <c r="F161" s="9" t="inlineStr">
+        <is>
+          <t>Meaning somebody graded it. I found the rubric. It's older than the city.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="7" t="inlineStr"/>
+      <c r="B162" s="6" t="inlineStr"/>
+      <c r="C162" s="7" t="inlineStr">
+        <is>
           <t>the Skilled Doctor</t>
         </is>
       </c>
-      <c r="D161" s="9" t="inlineStr">
+      <c r="D162" s="7" t="inlineStr">
         <is>
           <t>I'll get my good thread. Someone's getting stitches either way.</t>
         </is>
       </c>
-      <c r="E161" s="8" t="inlineStr">
+      <c r="E162" s="6" t="inlineStr">
         <is>
           <t>THE SKILLED DOCTOR</t>
         </is>
       </c>
-      <c r="F161" s="9" t="inlineStr">
+      <c r="F162" s="7" t="inlineStr">
         <is>
           <t>I'll get my good thread. Someone's getting stitches either way.</t>
         </is>
       </c>
     </row>
-    <row r="162">
-      <c r="A162" s="7" t="n">
+    <row r="163">
+      <c r="A163" s="9" t="n">
         <v>39</v>
       </c>
-      <c r="B162" s="6" t="inlineStr">
+      <c r="B163" s="8" t="inlineStr">
         <is>
           <t>Ascension Day</t>
         </is>
       </c>
-      <c r="C162" s="7" t="inlineStr">
+      <c r="C163" s="9" t="inlineStr">
         <is>
           <t>Timely Rain</t>
         </is>
       </c>
-      <c r="D162" s="7" t="inlineStr">
+      <c r="D163" s="9" t="inlineStr">
         <is>
           <t>Every kindness. Every bowl of soup. They wrote it before I meant it.</t>
         </is>
       </c>
-      <c r="E162" s="6" t="inlineStr">
+      <c r="E163" s="8" t="inlineStr">
         <is>
           <t>TIMELY RAIN</t>
         </is>
       </c>
-      <c r="F162" s="7" t="inlineStr">
+      <c r="F163" s="9" t="inlineStr">
         <is>
           <t>Every kindness. Every bowl of soup. They wrote it before I meant it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="9" t="inlineStr"/>
-      <c r="B163" s="8" t="inlineStr"/>
-      <c r="C163" s="9" t="inlineStr">
-        <is>
-          <t>the Tattooed Monk</t>
-        </is>
-      </c>
-      <c r="D163" s="9" t="inlineStr">
-        <is>
-          <t>You still meant it. Their pen, your hand. The soup was real, brother.</t>
-        </is>
-      </c>
-      <c r="E163" s="8" t="inlineStr">
-        <is>
-          <t>THE TATTOOED MONK</t>
-        </is>
-      </c>
-      <c r="F163" s="9" t="inlineStr">
-        <is>
-          <t>You still meant it. Their pen, your hand. The soup was real, brother.</t>
         </is>
       </c>
     </row>
@@ -26185,22 +26185,22 @@
       <c r="B164" s="6" t="inlineStr"/>
       <c r="C164" s="7" t="inlineStr">
         <is>
-          <t>Timely Rain</t>
+          <t>the Tattooed Monk</t>
         </is>
       </c>
       <c r="D164" s="7" t="inlineStr">
         <is>
-          <t>The ledger was the harvest list. I kept it FOR them.</t>
+          <t>You still meant it. Their pen, your hand. The soup was real, brother.</t>
         </is>
       </c>
       <c r="E164" s="6" t="inlineStr">
         <is>
-          <t>TIMELY RAIN</t>
+          <t>THE TATTOOED MONK</t>
         </is>
       </c>
       <c r="F164" s="7" t="inlineStr">
         <is>
-          <t>The ledger was the harvest list. I kept it FOR them.</t>
+          <t>You still meant it. Their pen, your hand. The soup was real, brother.</t>
         </is>
       </c>
     </row>
@@ -26209,76 +26209,76 @@
       <c r="B165" s="8" t="inlineStr"/>
       <c r="C165" s="9" t="inlineStr">
         <is>
+          <t>Timely Rain</t>
+        </is>
+      </c>
+      <c r="D165" s="9" t="inlineStr">
+        <is>
+          <t>The ledger was the harvest list. I kept it FOR them.</t>
+        </is>
+      </c>
+      <c r="E165" s="8" t="inlineStr">
+        <is>
+          <t>TIMELY RAIN</t>
+        </is>
+      </c>
+      <c r="F165" s="9" t="inlineStr">
+        <is>
+          <t>The ledger was the harvest list. I kept it FOR them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="7" t="inlineStr"/>
+      <c r="B166" s="6" t="inlineStr"/>
+      <c r="C166" s="7" t="inlineStr">
+        <is>
           <t>the Wisdom Star</t>
         </is>
       </c>
-      <c r="D165" s="9" t="inlineStr">
+      <c r="D166" s="7" t="inlineStr">
         <is>
           <t>Then we're the first crop to read the farmer's mail. Move. They know we know.</t>
         </is>
       </c>
-      <c r="E165" s="8" t="inlineStr">
+      <c r="E166" s="6" t="inlineStr">
         <is>
           <t>THE WISDOM STAR</t>
         </is>
       </c>
-      <c r="F165" s="9" t="inlineStr">
+      <c r="F166" s="7" t="inlineStr">
         <is>
           <t>Then we're the first crop to read the farmer's mail. Move. They know we know.</t>
         </is>
       </c>
     </row>
-    <row r="166">
-      <c r="A166" s="7" t="n">
+    <row r="167">
+      <c r="A167" s="9" t="n">
         <v>40</v>
       </c>
-      <c r="B166" s="6" t="inlineStr">
+      <c r="B167" s="8" t="inlineStr">
         <is>
           <t>The Harvest</t>
         </is>
       </c>
-      <c r="C166" s="7" t="inlineStr">
+      <c r="C167" s="9" t="inlineStr">
         <is>
           <t>Twin Rods</t>
         </is>
       </c>
-      <c r="D166" s="7" t="inlineStr">
+      <c r="D167" s="9" t="inlineStr">
         <is>
           <t>Marshals hold rearguards. It's the one order I'm keeping.</t>
         </is>
       </c>
-      <c r="E166" s="6" t="inlineStr">
+      <c r="E167" s="8" t="inlineStr">
         <is>
           <t>TWIN RODS</t>
         </is>
       </c>
-      <c r="F166" s="7" t="inlineStr">
+      <c r="F167" s="9" t="inlineStr">
         <is>
           <t>Marshals hold rearguards. It's the one order I'm keeping.</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="9" t="inlineStr"/>
-      <c r="B167" s="8" t="inlineStr"/>
-      <c r="C167" s="9" t="inlineStr">
-        <is>
-          <t>the Living Death-God</t>
-        </is>
-      </c>
-      <c r="D167" s="9" t="inlineStr">
-        <is>
-          <t>Race you to the bottom, marshal. Loser buys.</t>
-        </is>
-      </c>
-      <c r="E167" s="8" t="inlineStr">
-        <is>
-          <t>THE LIVING DEATH-GOD</t>
-        </is>
-      </c>
-      <c r="F167" s="9" t="inlineStr">
-        <is>
-          <t>Race you to the bottom, marshal. Loser buys.</t>
         </is>
       </c>
     </row>
@@ -26287,22 +26287,22 @@
       <c r="B168" s="6" t="inlineStr"/>
       <c r="C168" s="7" t="inlineStr">
         <is>
-          <t>Gold Lancer</t>
+          <t>the Living Death-God</t>
         </is>
       </c>
       <c r="D168" s="7" t="inlineStr">
         <is>
-          <t>Collar seams. Stairwell. Single file. Class dismissed. GO.</t>
+          <t>Race you to the bottom, marshal. Loser buys.</t>
         </is>
       </c>
       <c r="E168" s="6" t="inlineStr">
         <is>
-          <t>GOLD LANCER</t>
+          <t>THE LIVING DEATH-GOD</t>
         </is>
       </c>
       <c r="F168" s="7" t="inlineStr">
         <is>
-          <t>Collar seams. Stairwell. Single file. Class dismissed. GO.</t>
+          <t>Race you to the bottom, marshal. Loser buys.</t>
         </is>
       </c>
     </row>
@@ -26311,22 +26311,22 @@
       <c r="B169" s="8" t="inlineStr"/>
       <c r="C169" s="9" t="inlineStr">
         <is>
-          <t>Nine Dragons</t>
+          <t>Gold Lancer</t>
         </is>
       </c>
       <c r="D169" s="9" t="inlineStr">
         <is>
-          <t>We are not leaving them.</t>
+          <t>Collar seams. Stairwell. Single file. Class dismissed. GO.</t>
         </is>
       </c>
       <c r="E169" s="8" t="inlineStr">
         <is>
-          <t>NINE DRAGONS</t>
+          <t>GOLD LANCER</t>
         </is>
       </c>
       <c r="F169" s="9" t="inlineStr">
         <is>
-          <t>We are not leaving them.</t>
+          <t>Collar seams. Stairwell. Single file. Class dismissed. GO.</t>
         </is>
       </c>
     </row>
@@ -26335,76 +26335,76 @@
       <c r="B170" s="6" t="inlineStr"/>
       <c r="C170" s="7" t="inlineStr">
         <is>
+          <t>Nine Dragons</t>
+        </is>
+      </c>
+      <c r="D170" s="7" t="inlineStr">
+        <is>
+          <t>We are not leaving them.</t>
+        </is>
+      </c>
+      <c r="E170" s="6" t="inlineStr">
+        <is>
+          <t>NINE DRAGONS</t>
+        </is>
+      </c>
+      <c r="F170" s="7" t="inlineStr">
+        <is>
+          <t>We are not leaving them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="9" t="inlineStr"/>
+      <c r="B171" s="8" t="inlineStr"/>
+      <c r="C171" s="9" t="inlineStr">
+        <is>
           <t>Panther Head</t>
         </is>
       </c>
-      <c r="D170" s="7" t="inlineStr">
+      <c r="D171" s="9" t="inlineStr">
         <is>
           <t>We're not wasting them either. Run.</t>
         </is>
       </c>
-      <c r="E170" s="6" t="inlineStr">
+      <c r="E171" s="8" t="inlineStr">
         <is>
           <t>PANTHER HEAD</t>
         </is>
       </c>
-      <c r="F170" s="7" t="inlineStr">
+      <c r="F171" s="9" t="inlineStr">
         <is>
           <t>We're not wasting them either. Run.</t>
         </is>
       </c>
     </row>
-    <row r="171">
-      <c r="A171" s="9" t="n">
+    <row r="172">
+      <c r="A172" s="7" t="n">
         <v>41</v>
       </c>
-      <c r="B171" s="8" t="inlineStr">
+      <c r="B172" s="6" t="inlineStr">
         <is>
           <t>The Last Cup</t>
         </is>
       </c>
-      <c r="C171" s="9" t="inlineStr">
+      <c r="C172" s="7" t="inlineStr">
         <is>
           <t>Black Whirlwind</t>
         </is>
       </c>
-      <c r="D171" s="9" t="inlineStr">
+      <c r="D172" s="7" t="inlineStr">
         <is>
           <t>My plan has two steps now. Break the machine. Then the cup, together.</t>
         </is>
       </c>
-      <c r="E171" s="8" t="inlineStr">
+      <c r="E172" s="6" t="inlineStr">
         <is>
           <t>BLACK WHIRLWIND</t>
         </is>
       </c>
-      <c r="F171" s="9" t="inlineStr">
+      <c r="F172" s="7" t="inlineStr">
         <is>
           <t>My plan has two steps now. Break the machine. Then the cup, together.</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="7" t="inlineStr"/>
-      <c r="B172" s="6" t="inlineStr"/>
-      <c r="C172" s="7" t="inlineStr">
-        <is>
-          <t>Panther Head</t>
-        </is>
-      </c>
-      <c r="D172" s="7" t="inlineStr">
-        <is>
-          <t>Two steps. Look at you.</t>
-        </is>
-      </c>
-      <c r="E172" s="6" t="inlineStr">
-        <is>
-          <t>PANTHER HEAD</t>
-        </is>
-      </c>
-      <c r="F172" s="7" t="inlineStr">
-        <is>
-          <t>Two steps. Look at you.</t>
         </is>
       </c>
     </row>
@@ -26413,22 +26413,22 @@
       <c r="B173" s="8" t="inlineStr"/>
       <c r="C173" s="9" t="inlineStr">
         <is>
-          <t>Black Whirlwind</t>
+          <t>Panther Head</t>
         </is>
       </c>
       <c r="D173" s="9" t="inlineStr">
         <is>
-          <t>I saved the good plan for last.</t>
+          <t>Two steps. Look at you.</t>
         </is>
       </c>
       <c r="E173" s="8" t="inlineStr">
         <is>
-          <t>BLACK WHIRLWIND</t>
+          <t>PANTHER HEAD</t>
         </is>
       </c>
       <c r="F173" s="9" t="inlineStr">
         <is>
-          <t>I saved the good plan for last.</t>
+          <t>Two steps. Look at you.</t>
         </is>
       </c>
     </row>
@@ -26437,22 +26437,22 @@
       <c r="B174" s="6" t="inlineStr"/>
       <c r="C174" s="7" t="inlineStr">
         <is>
-          <t>Timely Rain</t>
+          <t>Black Whirlwind</t>
         </is>
       </c>
       <c r="D174" s="7" t="inlineStr">
         <is>
-          <t>Stand on my other side, brother. One last time.</t>
+          <t>I saved the good plan for last.</t>
         </is>
       </c>
       <c r="E174" s="6" t="inlineStr">
         <is>
-          <t>TIMELY RAIN</t>
+          <t>BLACK WHIRLWIND</t>
         </is>
       </c>
       <c r="F174" s="7" t="inlineStr">
         <is>
-          <t>Stand on my other side, brother. One last time.</t>
+          <t>I saved the good plan for last.</t>
         </is>
       </c>
     </row>
@@ -26461,76 +26461,76 @@
       <c r="B175" s="8" t="inlineStr"/>
       <c r="C175" s="9" t="inlineStr">
         <is>
+          <t>Timely Rain</t>
+        </is>
+      </c>
+      <c r="D175" s="9" t="inlineStr">
+        <is>
+          <t>Stand on my other side, brother. One last time.</t>
+        </is>
+      </c>
+      <c r="E175" s="8" t="inlineStr">
+        <is>
+          <t>TIMELY RAIN</t>
+        </is>
+      </c>
+      <c r="F175" s="9" t="inlineStr">
+        <is>
+          <t>Stand on my other side, brother. One last time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="7" t="inlineStr"/>
+      <c r="B176" s="6" t="inlineStr"/>
+      <c r="C176" s="7" t="inlineStr">
+        <is>
           <t>the Skilled Doctor</t>
         </is>
       </c>
-      <c r="D175" s="9" t="inlineStr">
+      <c r="D176" s="7" t="inlineStr">
         <is>
           <t>Everyone's stitched. Best work I ever did. Let's not waste it slowly.</t>
         </is>
       </c>
-      <c r="E175" s="8" t="inlineStr">
+      <c r="E176" s="6" t="inlineStr">
         <is>
           <t>THE SKILLED DOCTOR</t>
         </is>
       </c>
-      <c r="F175" s="9" t="inlineStr">
+      <c r="F176" s="7" t="inlineStr">
         <is>
           <t>Everyone's stitched. Best work I ever did. Let's not waste it slowly.</t>
         </is>
       </c>
     </row>
-    <row r="176">
-      <c r="A176" s="7" t="n">
+    <row r="177">
+      <c r="A177" s="9" t="n">
         <v>42</v>
       </c>
-      <c r="B176" s="6" t="inlineStr">
+      <c r="B177" s="8" t="inlineStr">
         <is>
           <t>Outer Heaven</t>
         </is>
       </c>
-      <c r="C176" s="7" t="inlineStr">
+      <c r="C177" s="9" t="inlineStr">
         <is>
           <t>Timely Rain</t>
         </is>
       </c>
-      <c r="D176" s="7" t="inlineStr">
+      <c r="D177" s="9" t="inlineStr">
         <is>
           <t>To the ones ahead. Keep the soup warm.</t>
         </is>
       </c>
-      <c r="E176" s="6" t="inlineStr">
+      <c r="E177" s="8" t="inlineStr">
         <is>
           <t>TIMELY RAIN</t>
         </is>
       </c>
-      <c r="F176" s="7" t="inlineStr">
+      <c r="F177" s="9" t="inlineStr">
         <is>
           <t>To the ones ahead. Keep the soup warm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="9" t="inlineStr"/>
-      <c r="B177" s="8" t="inlineStr"/>
-      <c r="C177" s="9" t="inlineStr">
-        <is>
-          <t>the Tattooed Monk</t>
-        </is>
-      </c>
-      <c r="D177" s="9" t="inlineStr">
-        <is>
-          <t>Final score: they predicted everything, and still lost. I counted.</t>
-        </is>
-      </c>
-      <c r="E177" s="8" t="inlineStr">
-        <is>
-          <t>THE TATTOOED MONK</t>
-        </is>
-      </c>
-      <c r="F177" s="9" t="inlineStr">
-        <is>
-          <t>Final score: they predicted everything, and still lost. I counted.</t>
         </is>
       </c>
     </row>
@@ -26539,22 +26539,22 @@
       <c r="B178" s="6" t="inlineStr"/>
       <c r="C178" s="7" t="inlineStr">
         <is>
-          <t>the Wanderer</t>
+          <t>the Tattooed Monk</t>
         </is>
       </c>
       <c r="D178" s="7" t="inlineStr">
         <is>
-          <t>Best angle I ever played was you people.</t>
+          <t>Final score: they predicted everything, and still lost. I counted.</t>
         </is>
       </c>
       <c r="E178" s="6" t="inlineStr">
         <is>
-          <t>THE WANDERER</t>
+          <t>THE TATTOOED MONK</t>
         </is>
       </c>
       <c r="F178" s="7" t="inlineStr">
         <is>
-          <t>Best angle I ever played was you people.</t>
+          <t>Final score: they predicted everything, and still lost. I counted.</t>
         </is>
       </c>
     </row>
@@ -26563,22 +26563,22 @@
       <c r="B179" s="8" t="inlineStr"/>
       <c r="C179" s="9" t="inlineStr">
         <is>
-          <t>Nine Dragons</t>
+          <t>the Wanderer</t>
         </is>
       </c>
       <c r="D179" s="9" t="inlineStr">
         <is>
-          <t>I believe the bedtime story now. Just not their version.</t>
+          <t>Best angle I ever played was you people.</t>
         </is>
       </c>
       <c r="E179" s="8" t="inlineStr">
         <is>
-          <t>NINE DRAGONS</t>
+          <t>THE WANDERER</t>
         </is>
       </c>
       <c r="F179" s="9" t="inlineStr">
         <is>
-          <t>I believe the bedtime story now. Just not their version.</t>
+          <t>Best angle I ever played was you people.</t>
         </is>
       </c>
     </row>
@@ -26587,20 +26587,44 @@
       <c r="B180" s="6" t="inlineStr"/>
       <c r="C180" s="7" t="inlineStr">
         <is>
+          <t>Nine Dragons</t>
+        </is>
+      </c>
+      <c r="D180" s="7" t="inlineStr">
+        <is>
+          <t>I believe the bedtime story now. Just not their version.</t>
+        </is>
+      </c>
+      <c r="E180" s="6" t="inlineStr">
+        <is>
+          <t>NINE DRAGONS</t>
+        </is>
+      </c>
+      <c r="F180" s="7" t="inlineStr">
+        <is>
+          <t>I believe the bedtime story now. Just not their version.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="9" t="inlineStr"/>
+      <c r="B181" s="8" t="inlineStr"/>
+      <c r="C181" s="9" t="inlineStr">
+        <is>
           <t>Timely Rain</t>
         </is>
       </c>
-      <c r="D180" s="7" t="inlineStr">
+      <c r="D181" s="9" t="inlineStr">
         <is>
           <t>Ours ends better. All together now.</t>
         </is>
       </c>
-      <c r="E180" s="6" t="inlineStr">
+      <c r="E181" s="8" t="inlineStr">
         <is>
           <t>TIMELY RAIN</t>
         </is>
       </c>
-      <c r="F180" s="7" t="inlineStr">
+      <c r="F181" s="9" t="inlineStr">
         <is>
           <t>Ours ends better. All together now.</t>
         </is>

</xml_diff>